<commit_message>
Sistema MCE: Actualización de matriz - 25-May-26 21:40
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,6 +513,47 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Acuerdos</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>25-May-26</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Jesus Morales</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>⚙️ Ingenieria</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>01-Jun-26</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sistema MCE: Actualización de matriz - 25-May-26 21:41
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -555,6 +555,47 @@
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
     </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Programa de Actividades</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>25-May-26</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Jesus Morales</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>⚙️ Ingenieria</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>01-Jun-26</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-05-26 23:20:28)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +25,35 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <color rgb="00000000"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00721C24"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D4EDDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8D7DA"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +68,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,7 +451,7 @@
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="25" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -487,372 +512,372 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>11-May-26</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>11-May-26</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>📦 Almacen</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>Elaborar calculo de material de lista entregada por Planeación planta Tableros.</t>
         </is>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>11-May-26</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>11-May-26</t>
+        </is>
+      </c>
+      <c r="J2" s="1" t="inlineStr">
         <is>
           <t>12/May - Solo enviar correo con resumen</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" s="1" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>11-May-26</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>11-May-26</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="1" t="inlineStr">
         <is>
           <t>Elaborar Ayuda visual de comandos en maquinas Láser</t>
         </is>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="1" t="inlineStr">
         <is>
           <t>15-May-26</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="J3" s="1" t="inlineStr"/>
+      <c r="K3" s="1" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>11-May-26</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>11-May-26</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Capacitar a personal nuevo ingreso Flores Campa Marvin Manuel</t>
         </is>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>11-May-26</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>11-May-26</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Capacitar a personal nuevo ingreso Campos Martinez Jesus Manuel</t>
         </is>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>11-May-26</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>11-May-26</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>✂️ Corte</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="1" t="inlineStr">
         <is>
           <t>Hacer pruebas de corte de Cobre</t>
         </is>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" s="1" t="inlineStr">
         <is>
           <t>15-May-26</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="J6" s="1" t="inlineStr"/>
+      <c r="K6" s="1" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>11-May-26</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>11-May-26</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Capacitar a personal nuevo ingreso Alejandro Hernandez Perez</t>
         </is>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>Mejoras</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>11-May-26</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>11-May-26</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="1" t="inlineStr">
         <is>
           <t>✂️ Corte</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="1" t="inlineStr">
         <is>
           <t>Elaborar Mesas de Cortadora</t>
         </is>
       </c>
-      <c r="H8" t="n">
+      <c r="H8" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I8" s="1" t="inlineStr">
         <is>
           <t>15-May-26</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="J8" s="1" t="inlineStr"/>
+      <c r="K8" s="1" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>11-May-26</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>11-May-26</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="1" t="inlineStr">
         <is>
           <t>📐 Doblez</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" s="1" t="inlineStr">
         <is>
           <t>Revisar herramental de FLEX</t>
         </is>
       </c>
-      <c r="H9" t="n">
+      <c r="H9" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I9" s="1" t="inlineStr">
         <is>
           <t>15-May-26</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J9" s="1" t="inlineStr">
         <is>
           <t>12/May - Falto las Matrices ya se comunico con COMPRAS</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
+      <c r="K9" s="1" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1035,466 +1060,466 @@
       <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Mejoras</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>11-May-26</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>11-May-26</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>📐 Doblez</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Cotizar Refacciones de maquinas Dobladoras</t>
         </is>
       </c>
-      <c r="H14" t="n">
+      <c r="H14" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>12/May - Se mando Correo a Flex con Imágenes</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>Mejoras</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>11-May-26</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>11-May-26</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F15" s="1" t="inlineStr">
         <is>
           <t>📐 Doblez</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G15" s="1" t="inlineStr">
         <is>
           <t>Investigación de cursos ó DC3 para operadores de Doblez</t>
         </is>
       </c>
-      <c r="H15" t="n">
+      <c r="H15" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I15" s="1" t="inlineStr">
         <is>
           <t>22-May-26</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="J15" s="1" t="inlineStr">
         <is>
           <t>Mande correo https://agentes.stps.gob.mx/</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
+      <c r="K15" s="1" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" s="1" t="n">
         <v>15</v>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>11-May-26</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>11-May-26</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>Luis Quintana</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F16" s="1" t="inlineStr">
         <is>
           <t>🎨 Pintura</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G16" s="1" t="inlineStr">
         <is>
           <t>Investigación de curso para pintura VITRACOAT</t>
         </is>
       </c>
-      <c r="H16" t="n">
+      <c r="H16" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I16" s="1" t="inlineStr">
         <is>
           <t>14-May-26</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J16" s="1" t="inlineStr">
         <is>
           <t>15/May - Capacitación y revisión en GALVATEK</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
+      <c r="K16" s="1" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>11-May-26</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>11-May-26</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
         <is>
           <t>Luis Quintana</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="1" t="inlineStr">
         <is>
           <t>🎨 Pintura</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" s="1" t="inlineStr">
         <is>
           <t>Elaboración manual de capacitación de operadores de pintura</t>
         </is>
       </c>
-      <c r="H17" t="n">
+      <c r="H17" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I17" s="1" t="inlineStr">
         <is>
           <t>14-May-26</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="J17" s="1" t="inlineStr"/>
+      <c r="K17" s="1" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="n">
+      <c r="A18" s="1" t="n">
         <v>17</v>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>11-May-26</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t>11-May-26</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="inlineStr">
         <is>
           <t>URGENT</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="1" t="inlineStr">
         <is>
           <t>Luis Quintana</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>🎨 Pintura</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G18" s="1" t="inlineStr">
         <is>
           <t>Elaborar inventario de Faltantes ó Reposiciones</t>
         </is>
       </c>
-      <c r="H18" t="n">
+      <c r="H18" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="I18" s="1" t="inlineStr">
         <is>
           <t>13-May-26</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+      <c r="J18" s="1" t="inlineStr"/>
+      <c r="K18" s="1" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="n">
+      <c r="A19" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>11-May-26</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>11-May-26</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="inlineStr">
         <is>
           <t>URGENT</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>Luis Quintana</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>🎨 Pintura</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G19" s="1" t="inlineStr">
         <is>
           <t>Elaborar Layout de Planta Pintura</t>
         </is>
       </c>
-      <c r="H19" t="n">
+      <c r="H19" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I19" s="1" t="inlineStr">
         <is>
           <t>15-May-26</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
+      <c r="J19" s="1" t="inlineStr"/>
+      <c r="K19" s="1" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="n">
+      <c r="A20" s="1" t="n">
         <v>19</v>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>11-May-26</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>11-May-26</t>
+        </is>
+      </c>
+      <c r="D20" s="1" t="inlineStr">
         <is>
           <t>URGENT</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="1" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>⚙️ Ingenieria</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" s="1" t="inlineStr">
         <is>
           <t>Elaborar Perfil de puesto de Jefe de Embarques</t>
         </is>
       </c>
-      <c r="H20" t="n">
+      <c r="H20" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I20" s="1" t="inlineStr">
         <is>
           <t>13-May-26</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="J20" s="1" t="inlineStr"/>
+      <c r="K20" s="1" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" t="n">
+      <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Auto Asignado</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>11-May-26</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>11-May-26</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>⚙️ Ingenieria</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>Autorización compra de aspiradora para limpieza de Lijadora</t>
         </is>
       </c>
-      <c r="H21" t="n">
+      <c r="H21" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="n">
+      <c r="A22" s="1" t="n">
         <v>21</v>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>Auto Asignado</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>11-May-26</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>11-May-26</t>
+        </is>
+      </c>
+      <c r="D22" s="1" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F22" s="1" t="inlineStr">
         <is>
           <t>⚙️ Ingenieria</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G22" s="1" t="inlineStr">
         <is>
           <t>Fabricación de Uñas para montacargas</t>
         </is>
       </c>
-      <c r="H22" t="n">
+      <c r="H22" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="I22" s="1" t="inlineStr">
         <is>
           <t>14-May-26</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="J22" s="1" t="inlineStr"/>
+      <c r="K22" s="1" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="n">
+      <c r="A23" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="1" t="inlineStr">
         <is>
           <t>12-May-26</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
+      <c r="D23" s="1" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F23" s="1" t="inlineStr">
         <is>
           <t>⚙️ Ingenieria</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G23" s="1" t="inlineStr">
         <is>
           <t>Autorización de Compra de Banda de transportador de Lijadora</t>
         </is>
       </c>
-      <c r="H23" t="n">
+      <c r="H23" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I23" s="1" t="inlineStr">
         <is>
           <t>15-May-26</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
+      <c r="J23" s="1" t="inlineStr"/>
+      <c r="K23" s="1" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1542,49 +1567,49 @@
       <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" t="n">
+      <c r="A25" s="1" t="n">
         <v>24</v>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="1" t="inlineStr">
         <is>
           <t>Problema de Seguridad</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="1" t="inlineStr">
         <is>
           <t>12-May-26</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="1" t="inlineStr">
         <is>
           <t>URGENT</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="1" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F25" s="1" t="inlineStr">
         <is>
           <t>⚙️ Ingenieria</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G25" s="1" t="inlineStr">
         <is>
           <t>Autorización de Material para Botiquin Primeros Auxilios</t>
         </is>
       </c>
-      <c r="H25" t="n">
+      <c r="H25" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="I25" s="1" t="inlineStr">
         <is>
           <t>12-May-26</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
+      <c r="J25" s="1" t="inlineStr"/>
+      <c r="K25" s="1" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1632,49 +1657,49 @@
       <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="n">
+      <c r="A27" s="1" t="n">
         <v>26</v>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="1" t="inlineStr">
         <is>
           <t>12-May-26</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
+      <c r="D27" s="1" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E27" s="1" t="inlineStr">
         <is>
           <t>Luis Quintana</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F27" s="1" t="inlineStr">
         <is>
           <t>🚚 Embarquez</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G27" s="1" t="inlineStr">
         <is>
           <t>Garantia de reposición PNC-2554</t>
         </is>
       </c>
-      <c r="H27" t="n">
+      <c r="H27" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="I27" s="1" t="inlineStr">
         <is>
           <t>12-May-26</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
+      <c r="J27" s="1" t="inlineStr"/>
+      <c r="K27" s="1" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1722,98 +1747,98 @@
       <c r="K28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" t="n">
+      <c r="A29" s="1" t="n">
         <v>28</v>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="1" t="inlineStr">
         <is>
           <t>Dirección</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="1" t="inlineStr">
         <is>
           <t>18-May-26</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="1" t="inlineStr">
         <is>
           <t>URGENT</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" s="1" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F29" s="1" t="inlineStr">
         <is>
           <t>🚚 Embarquez</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G29" s="1" t="inlineStr">
         <is>
           <t>Elaborar Solicitud de Movimiento de personal para Jefe de Empaque y Logistica</t>
         </is>
       </c>
-      <c r="H29" t="n">
+      <c r="H29" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="I29" s="1" t="inlineStr">
         <is>
           <t>18-May-26</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="J29" s="1" t="inlineStr">
         <is>
           <t>18/May - Enfiado a Autorización</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
+      <c r="K29" s="1" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" t="n">
+      <c r="A30" s="1" t="n">
         <v>29</v>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="1" t="inlineStr">
         <is>
           <t>Dirección</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="1" t="inlineStr">
         <is>
           <t>18-May-26</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="1" t="inlineStr">
         <is>
           <t>URGENT</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E30" s="1" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F30" s="1" t="inlineStr">
         <is>
           <t>🏭 Planta Rio</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G30" s="1" t="inlineStr">
         <is>
           <t>Detener el proceso de Fabricación Cal 12 con espesore bajo</t>
         </is>
       </c>
-      <c r="H30" t="n">
+      <c r="H30" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="I30" s="1" t="inlineStr">
         <is>
           <t>18-May-26</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
+      <c r="J30" s="1" t="inlineStr"/>
+      <c r="K30" s="1" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1861,204 +1886,190 @@
       <c r="K31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" t="n">
+      <c r="A32" s="1" t="n">
         <v>31</v>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="1" t="inlineStr">
         <is>
           <t>Acuerdos</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="1" t="inlineStr">
         <is>
           <t>18-May-26</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="1" t="inlineStr">
         <is>
           <t>URGENT</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" s="1" t="inlineStr">
         <is>
           <t>Luis Quintana</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F32" s="1" t="inlineStr">
         <is>
           <t>📦 Almacen</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G32" s="1" t="inlineStr">
         <is>
           <t>Inventario 19/May - Galvatek</t>
         </is>
       </c>
-      <c r="H32" t="n">
+      <c r="H32" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="I32" s="1" t="inlineStr">
         <is>
           <t>19-Feb-26</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
+      <c r="J32" s="1" t="inlineStr"/>
+      <c r="K32" s="1" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" t="n">
+      <c r="A33" s="1" t="n">
         <v>32</v>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="1" t="inlineStr">
         <is>
           <t>Acuerdos</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="1" t="inlineStr">
         <is>
           <t>18-May-26</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="1" t="inlineStr">
         <is>
           <t>URGENT</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="1" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F33" s="1" t="inlineStr">
         <is>
           <t>📦 Almacen</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G33" s="1" t="inlineStr">
         <is>
           <t>Inventario 19/May - Sigrama Diagonal</t>
         </is>
       </c>
-      <c r="H33" t="n">
+      <c r="H33" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="I33" s="1" t="inlineStr">
         <is>
           <t>19-Feb-26</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
+      <c r="J33" s="1" t="inlineStr"/>
+      <c r="K33" s="1" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" t="n">
+      <c r="A34" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>25-May-26</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
         <is>
           <t>Luis Quintana</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F34" s="3" t="inlineStr">
         <is>
           <t>📦 Almacen</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t>Requisición de Quimicos para lineas de Pintura</t>
         </is>
       </c>
-      <c r="H34" t="n">
+      <c r="H34" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="I34" s="3" t="inlineStr">
         <is>
           <t>26-May-26</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="J34" s="3" t="inlineStr">
         <is>
           <t>25/May - Hacer la Lista de Quimicos a cotizar con COATEK para darlos de Alta en SIGRAMA</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr"/>
+      <c r="K34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="n">
+      <c r="A35" s="3" t="n">
         <v>34</v>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>Auto Asignado</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>25-May-26</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>NORMAL</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>📦 Almacen</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>Solicitud de Computadora para Rodolfo Ingenieria</t>
         </is>
       </c>
-      <c r="H35" t="n">
+      <c r="H35" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="I35" s="3" t="inlineStr">
         <is>
           <t>26-May-26</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
+      <c r="J35" s="3" t="inlineStr"/>
+      <c r="K35" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="4">
-    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Acuerdos,Programa de Actividades,Actividades Sujeridas,Dirección,Problema de Calidad,Problema de Seguridad,Lista de Pendientes,Auto Asignado,Plan de Control y Monitoreo,Mejoras,Investigación,Manuales,Procesos"</formula1>
-    </dataValidation>
-    <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Baja,Media,Urgente"</formula1>
-    </dataValidation>
-    <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Jesus Morales,Ing. Alfredo Hdz,Ing. Lorena Hdz,Jesús Alday,Alejandra Arellano,Jose Romo,Jose Manuel Aldama,Fernando Llanas,Celso,Cruz Carreon,Luis Quintana,Bryan Flores,Jorge Sanchez,Voctor Montoya,Moises Hernandez,Rodolfo Ferndez M"</formula1>
-    </dataValidation>
-    <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"⚙️ Ingenieria,🔍 Calidad,📦 Almacen,✂️ Corte,📐 Doblez,🎨 Pintura,🚚 Embarquez,🏭 Planta Rio"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-05-26 23:21:43)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:K45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1811,7 +1811,7 @@
       </c>
       <c r="D30" s="1" t="inlineStr">
         <is>
-          <t>URGENT</t>
+          <t>Urgente</t>
         </is>
       </c>
       <c r="E30" s="1" t="inlineStr">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>URGENT</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="D32" s="1" t="inlineStr">
         <is>
-          <t>URGENT</t>
+          <t>Urgente</t>
         </is>
       </c>
       <c r="E32" s="1" t="inlineStr">
@@ -1946,7 +1946,7 @@
       </c>
       <c r="D33" s="1" t="inlineStr">
         <is>
-          <t>URGENT</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E33" s="1" t="inlineStr">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -2040,7 +2040,7 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
@@ -2068,6 +2068,460 @@
       </c>
       <c r="J35" s="3" t="inlineStr"/>
       <c r="K35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Dirección</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2026-05-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Jesus Morales</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>📐 Doblez</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Capacitar en sistema SAI para hacer Requisiciones en Sistema.</t>
+        </is>
+      </c>
+      <c r="H36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>2026-05-29 00:00:00</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Programa de Actividades</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2026-05-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Cruz Carreon</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>✂️ Corte</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Fabricar mesas para Tarimas con material reciclado, Altura ergonomica</t>
+        </is>
+      </c>
+      <c r="H37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>2026-05-29 00:00:00</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Programa de Actividades</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2026-05-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Bryan Flores</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>✂️ Corte</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Delimitar area de precausion de Maquina Lijadora (Negro-Amarillo)</t>
+        </is>
+      </c>
+      <c r="H38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Programa de Actividades</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2026-05-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>🚚 Embarquez</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Presentar a Cruz y Bryan en planta RIO</t>
+        </is>
+      </c>
+      <c r="H39" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>2026-05-29 00:00:00</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Programa de Actividades</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2026-05-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Bryan Flores</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>✂️ Corte</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Instalar el Pintarron de Actividades de Planta Metales</t>
+        </is>
+      </c>
+      <c r="H40" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>2026-05-29 00:00:00</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Mejoras</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>2026-05-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Bryan Flores</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>⚙️ Ingenieria</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Capacitar en el uso de PRONEST</t>
+        </is>
+      </c>
+      <c r="H41" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2026-06-19 00:00:00</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Programa de Actividades</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>2026-05-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Jesus Morales</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>⚙️ Ingenieria</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Licencia PRONEST final</t>
+        </is>
+      </c>
+      <c r="H42" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>2026-06-19 00:00:00</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Programa de Actividades</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>2026-05-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Cruz Carreon</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>✂️ Corte</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Hacer Nuevo Organigrama de Personal</t>
+        </is>
+      </c>
+      <c r="H43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>2026-06-05 00:00:00</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Procesos</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>2026-05-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Bryan Flores</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>✂️ Corte</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Elaborar Procedimiento de Manufactura de Corte Laser.</t>
+        </is>
+      </c>
+      <c r="H44" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>2026-06-19 00:00:00</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Mejoras</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>2026-05-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Jesus Morales</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>⚙️ Ingenieria</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Solicitar tablets para el área de doblado y embarque.</t>
+        </is>
+      </c>
+      <c r="H45" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-05-26 23:24:27)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -527,7 +527,7 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
@@ -576,7 +576,7 @@
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
@@ -621,7 +621,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -711,7 +711,7 @@
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -801,7 +801,7 @@
       </c>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="E8" s="1" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="D9" s="1" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="E9" s="1" t="inlineStr">
@@ -895,7 +895,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -985,7 +985,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1124,7 +1124,7 @@
       </c>
       <c r="D15" s="1" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E15" s="1" t="inlineStr">
@@ -1173,7 +1173,7 @@
       </c>
       <c r="D16" s="1" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="E16" s="1" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="D17" s="1" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E17" s="1" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="D18" s="1" t="inlineStr">
         <is>
-          <t>URGENT</t>
+          <t>Urgente</t>
         </is>
       </c>
       <c r="E18" s="1" t="inlineStr">
@@ -1312,7 +1312,7 @@
       </c>
       <c r="D19" s="1" t="inlineStr">
         <is>
-          <t>URGENT</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E19" s="1" t="inlineStr">
@@ -1357,7 +1357,7 @@
       </c>
       <c r="D20" s="1" t="inlineStr">
         <is>
-          <t>URGENT</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E20" s="1" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1447,7 +1447,7 @@
       </c>
       <c r="D22" s="1" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="E22" s="1" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="D23" s="1" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E23" s="1" t="inlineStr">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="D25" s="1" t="inlineStr">
         <is>
-          <t>URGENT</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="E25" s="1" t="inlineStr">
@@ -1627,7 +1627,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1672,7 +1672,7 @@
       </c>
       <c r="D27" s="1" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Urgente</t>
         </is>
       </c>
       <c r="E27" s="1" t="inlineStr">
@@ -1717,7 +1717,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>NORMAL</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="D29" s="1" t="inlineStr">
         <is>
-          <t>URGENT</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E29" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-05-27 00:28:46)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -1383,8 +1383,16 @@
           <t>13-May-26</t>
         </is>
       </c>
-      <c r="J20" s="1" t="inlineStr"/>
-      <c r="K20" s="1" t="inlineStr"/>
+      <c r="J20" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K20" s="1" t="inlineStr">
+        <is>
+          <t>evidencias/MCE-019_evidencia.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-05-28 14:24:49)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -1383,11 +1383,7 @@
           <t>13-May-26</t>
         </is>
       </c>
-      <c r="J20" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="J20" s="1" t="inlineStr"/>
       <c r="K20" s="1" t="inlineStr">
         <is>
           <t>evidencias/MCE-019_evidencia.jpg</t>
@@ -2206,14 +2202,18 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
           <t>2026-05-28 00:00:00</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quedamos a espera de la llegada de pintura color Negro/Amarillo </t>
+        </is>
+      </c>
       <c r="K38" t="inlineStr"/>
     </row>
     <row r="39">
@@ -2262,49 +2262,49 @@
       <c r="K39" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" t="n">
+      <c r="A40" s="1" t="n">
         <v>39</v>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="1" t="inlineStr">
         <is>
           <t>2026-05-26 00:00:00</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
+      <c r="D40" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E40" s="1" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F40" s="1" t="inlineStr">
         <is>
           <t>✂️ Corte</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="G40" s="1" t="inlineStr">
         <is>
           <t>Instalar el Pintarron de Actividades de Planta Metales</t>
         </is>
       </c>
-      <c r="H40" t="n">
-        <v>0</v>
-      </c>
-      <c r="I40" t="inlineStr">
+      <c r="H40" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I40" s="1" t="inlineStr">
         <is>
           <t>2026-05-29 00:00:00</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
+      <c r="J40" s="1" t="inlineStr"/>
+      <c r="K40" s="1" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-05-28 15:03:30)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -2084,7 +2084,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-05-26 00:00:00</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-05-29 00:00:00</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-05-26 00:00:00</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2161,7 +2161,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-05-29 00:00:00</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="J37" t="inlineStr"/>
@@ -2178,7 +2178,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-05-26 00:00:00</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-05-28 00:00:00</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -2227,7 +2227,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-05-26 00:00:00</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2255,7 +2255,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-05-29 00:00:00</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="J39" t="inlineStr"/>
@@ -2272,7 +2272,7 @@
       </c>
       <c r="C40" s="1" t="inlineStr">
         <is>
-          <t>2026-05-26 00:00:00</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="D40" s="1" t="inlineStr">
@@ -2300,7 +2300,7 @@
       </c>
       <c r="I40" s="1" t="inlineStr">
         <is>
-          <t>2026-05-29 00:00:00</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="J40" s="1" t="inlineStr"/>
@@ -2317,7 +2317,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-05-26 00:00:00</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-06-19 00:00:00</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="J41" t="inlineStr"/>
@@ -2362,7 +2362,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026-05-26 00:00:00</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2390,7 +2390,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-06-19 00:00:00</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="J42" t="inlineStr"/>
@@ -2407,7 +2407,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026-05-26 00:00:00</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2435,7 +2435,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-06-05 00:00:00</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="J43" t="inlineStr"/>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-05-26 00:00:00</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-06-19 00:00:00</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="J44" t="inlineStr"/>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-05-26 00:00:00</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2525,7 +2525,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-06-12 00:00:00</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="J45" t="inlineStr"/>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-05-28 16:10:54)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -1980,53 +1980,53 @@
       <c r="K33" s="1" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="n">
+      <c r="A34" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>25-May-26</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>Luis Quintana</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>📦 Almacen</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>Requisición de Quimicos para lineas de Pintura</t>
         </is>
       </c>
-      <c r="H34" s="3" t="n">
+      <c r="H34" t="n">
         <v>0</v>
       </c>
-      <c r="I34" s="3" t="inlineStr">
-        <is>
-          <t>26-May-26</t>
-        </is>
-      </c>
-      <c r="J34" s="3" t="inlineStr">
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
         <is>
           <t>25/May - Hacer la Lista de Quimicos a cotizar con COATEK para darlos de Alta en SIGRAMA</t>
         </is>
       </c>
-      <c r="K34" s="3" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-05-28 16:11:58)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,12 +28,8 @@
     <font>
       <color rgb="00000000"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00721C24"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -50,11 +46,6 @@
         <fgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F8D7DA"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -68,11 +59,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2029,49 +2019,49 @@
       <c r="K34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="n">
+      <c r="A35" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>Auto Asignado</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>25-May-26</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>📦 Almacen</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>Solicitud de Computadora para Rodolfo Ingenieria</t>
         </is>
       </c>
-      <c r="H35" s="3" t="n">
+      <c r="H35" t="n">
         <v>0</v>
       </c>
-      <c r="I35" s="3" t="inlineStr">
-        <is>
-          <t>26-May-26</t>
-        </is>
-      </c>
-      <c r="J35" s="3" t="inlineStr"/>
-      <c r="K35" s="3" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>5-Jun-2029</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-05-28 17:20:25)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -1716,7 +1716,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Jesus Morales</t>
+          <t>Cruz Carreon</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1855,7 +1855,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Jesus Morales</t>
+          <t>Cruz Carreon</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-05-28 18:56:41)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -2207,49 +2207,57 @@
       <c r="K38" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" t="n">
+      <c r="A39" s="1" t="n">
         <v>38</v>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="1" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="1" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E39" s="1" t="inlineStr">
         <is>
           <t>Luis Quintana</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F39" s="1" t="inlineStr">
         <is>
           <t>🚚 Embarquez</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="G39" s="1" t="inlineStr">
         <is>
           <t>Presentar a Cruz y Bryan en planta RIO Area de Compras</t>
         </is>
       </c>
-      <c r="H39" t="n">
-        <v>0</v>
-      </c>
-      <c r="I39" t="inlineStr">
+      <c r="H39" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I39" s="1" t="inlineStr">
         <is>
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
+      <c r="J39" s="1" t="inlineStr">
+        <is>
+          <t>26/Mayo - Presento a Bryan (No se pueden ir los 3 al mismo tiempo).</t>
+        </is>
+      </c>
+      <c r="K39" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -2376,15 +2384,23 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>28/May - Hable con Cesar Campos (Ya llego a Monclova la van a mandar por paqueteria).</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-05-28 19:49:54)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -2053,15 +2053,23 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
           <t>5-Jun-2026</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>28/May - Solicitud eviada al Ing. Alfredo de PC para Ing. Rodolfo.</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2253,11 +2261,7 @@
           <t>26/Mayo - Presento a Bryan (No se pueden ir los 3 al mismo tiempo).</t>
         </is>
       </c>
-      <c r="K39" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K39" s="1" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -2396,11 +2400,7 @@
           <t>28/May - Hable con Cesar Campos (Ya llego a Monclova la van a mandar por paqueteria).</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2531,7 +2531,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="J45" t="inlineStr"/>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-05-28 19:57:09)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -1406,7 +1406,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>⚙️ Ingenieria</t>
+          <t>👑 Direccion</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1496,7 +1496,7 @@
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>⚙️ Ingenieria</t>
+          <t>👑 Direccion</t>
         </is>
       </c>
       <c r="G23" s="1" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>⚙️ Ingenieria</t>
+          <t>👑 Direccion</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>⚙️ Ingenieria</t>
+          <t>👑 Direccion</t>
         </is>
       </c>
       <c r="G25" s="1" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>⚙️ Ingenieria</t>
+          <t>👑 Direccion</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>📦 Almacen</t>
+          <t>👑 Direccion</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2097,7 +2097,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>📐 Doblez</t>
+          <t>👑 Direccion</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2518,7 +2518,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>⚙️ Ingenieria</t>
+          <t>👑 Direccion</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-05-28 20:13:33)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K45"/>
+  <dimension ref="A1:K46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2215,53 +2215,57 @@
       <c r="K38" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="1" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C39" s="1" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="D39" s="1" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E39" s="1" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>Luis Quintana</t>
         </is>
       </c>
-      <c r="F39" s="1" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>🚚 Embarquez</t>
         </is>
       </c>
-      <c r="G39" s="1" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>Presentar a Cruz y Bryan en planta RIO Area de Compras</t>
         </is>
       </c>
-      <c r="H39" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="I39" s="1" t="inlineStr">
+      <c r="H39" t="n">
+        <v>90</v>
+      </c>
+      <c r="I39" t="inlineStr">
         <is>
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="J39" s="1" t="inlineStr">
+      <c r="J39" t="inlineStr">
         <is>
           <t>26/Mayo - Presento a Bryan (No se pueden ir los 3 al mismo tiempo).</t>
         </is>
       </c>
-      <c r="K39" s="1" t="inlineStr"/>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -2536,6 +2540,51 @@
       </c>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Programa de Actividades</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>28-May-26</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>🚚 Embarquez</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>26/May  - Comenzar el proceso de empaquetado del Material en DIAGONAL 1600 piezas</t>
+        </is>
+      </c>
+      <c r="H46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>29-May-26</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-05-28 21:05:41)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -1238,8 +1238,16 @@
           <t>14-May-26</t>
         </is>
       </c>
-      <c r="J17" s="1" t="inlineStr"/>
-      <c r="K17" s="1" t="inlineStr"/>
+      <c r="J17" s="1" t="inlineStr">
+        <is>
+          <t>16/May - Terminado</t>
+        </is>
+      </c>
+      <c r="K17" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -1283,8 +1291,16 @@
           <t>13-May-26</t>
         </is>
       </c>
-      <c r="J18" s="1" t="inlineStr"/>
-      <c r="K18" s="1" t="inlineStr"/>
+      <c r="J18" s="1" t="inlineStr">
+        <is>
+          <t>21/May - Terminado y mandado correo a Equipo de Compras</t>
+        </is>
+      </c>
+      <c r="K18" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -1422,8 +1438,16 @@
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr"/>
-      <c r="K21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>26/May - Requisición en SAI  21396 - REQ. HTA. PARTE 2JM</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -1516,49 +1540,57 @@
       <c r="K23" s="1" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" t="n">
+      <c r="A24" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>12-May-26</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>👑 Direccion</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>Autorización de Matriz Dobladora 85x85x3200</t>
         </is>
       </c>
-      <c r="H24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" t="inlineStr">
+      <c r="H24" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">26/May - Requisición Aun no se tiene autorización 21485 - HERRAMENTAL DOBLEZ </t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -1647,8 +1679,16 @@
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>28/May - Se a reenviado las Requisiciones al Ing. Alfredo para autorización 21348-21092</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -2004,7 +2044,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -2013,10 +2053,14 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>25/May - Hacer la Lista de Quimicos a cotizar con COATEK para darlos de Alta en SIGRAMA</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr"/>
+          <t>28/May - Pendiente modificar Requi.   Con Numeros Articulos nuevos</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2115,10 +2159,14 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>...</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr"/>
+          <t>28/May - Se programa para Viernes 29 a las 10:00 a,m,</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2258,7 +2306,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>26/Mayo - Presento a Bryan (No se pueden ir los 3 al mismo tiempo).</t>
+          <t>26/Mayo - Presento a Bryan (No se pueden ir los 3 al mismo tiempo). Se programara visita cruz despues..!!!</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2538,53 +2586,65 @@
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>En investigación...!!!</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" t="n">
+      <c r="A46" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>28-May-26</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>Luis Quintana</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>🚚 Embarquez</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>26/May  - Comenzar el proceso de empaquetado del Material en DIAGONAL 1600 piezas</t>
         </is>
       </c>
-      <c r="H46" t="n">
-        <v>0</v>
-      </c>
-      <c r="I46" t="inlineStr">
+      <c r="H46" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
         <is>
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>28/May - 26 Tarimas Preparadas Apro 35% avance  1 Dia despues</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-05-28 23:28:34)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K46"/>
+  <dimension ref="A1:K49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -870,139 +870,151 @@
       <c r="K9" s="1" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Capacitar a personal nuevo ingreso Garcia Montoya Uriel Alejandro</t>
         </is>
       </c>
-      <c r="H10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" t="inlineStr">
+      <c r="H10" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Capacitar a personal nuevo ingreso Alvarado Rojas Miguel Antonio</t>
         </is>
       </c>
-      <c r="H11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" t="inlineStr">
+      <c r="H11" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Capacitar a personal nuevo ingreso Alvarado Aguilar Luis Alejandro</t>
         </is>
       </c>
-      <c r="H12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" t="inlineStr">
+      <c r="H12" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1084,7 +1096,7 @@
         </is>
       </c>
       <c r="H14" s="2" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
@@ -1096,7 +1108,11 @@
           <t>12/May - Se mando Correo a Flex con Imágenes</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -1243,11 +1259,7 @@
           <t>16/May - Terminado</t>
         </is>
       </c>
-      <c r="K17" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K17" s="1" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -1296,11 +1308,7 @@
           <t>21/May - Terminado y mandado correo a Equipo de Compras</t>
         </is>
       </c>
-      <c r="K18" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K18" s="1" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -1443,11 +1451,7 @@
           <t>26/May - Requisición en SAI  21396 - REQ. HTA. PARTE 2JM</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -1586,11 +1590,7 @@
           <t xml:space="preserve">26/May - Requisición Aun no se tiene autorización 21485 - HERRAMENTAL DOBLEZ </t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -1638,53 +1638,53 @@
       <c r="K25" s="1" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" t="n">
+      <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>12-May-26</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>👑 Direccion</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>Autorización de Escritorios y Sillas</t>
         </is>
       </c>
-      <c r="H26" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" t="inlineStr">
+      <c r="H26" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
         <is>
           <t>28/May - Se a reenviado las Requisiciones al Ing. Alfredo para autorización 21348-21092</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
@@ -2056,11 +2056,7 @@
           <t>28/May - Pendiente modificar Requi.   Con Numeros Articulos nuevos</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2109,11 +2105,7 @@
           <t>28/May - Solicitud eviada al Ing. Alfredo de PC para Ing. Rodolfo.</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2162,11 +2154,7 @@
           <t>28/May - Se programa para Viernes 29 a las 10:00 a,m,</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2309,11 +2297,7 @@
           <t>26/Mayo - Presento a Bryan (No se pueden ir los 3 al mismo tiempo). Se programara visita cruz despues..!!!</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -2440,7 +2424,7 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
@@ -2452,7 +2436,11 @@
           <t>28/May - Hable con Cesar Campos (Ya llego a Monclova la van a mandar por paqueteria).</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2489,15 +2477,23 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
           <t>2026-06-05</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>28/May - Ajustando con el Organigrama oficial la actividad es separar al personal.</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2591,11 +2587,7 @@
           <t>En investigación...!!!</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -2645,6 +2637,141 @@
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Dirección</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>28-May-26</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>📦 Almacen</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Reubicar los racks a la pared bajo el Extractor.</t>
+        </is>
+      </c>
+      <c r="H47" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>05-Jun-26</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Programa de Actividades</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>28-May-26</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Rodolfo Ferndez M</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>⚙️ Ingenieria</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Elaborar el primer procedimiento de Ingenieria para primera pieza segén el proceso actual</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>05-Jun-26</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr"/>
+      <c r="K48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Programa de Actividades</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>28-May-26</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Rodolfo Ferndez M</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>⚙️ Ingenieria</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Hacer 10 planos con las correcciones solicitadas por departamento de Calidad para estresar procedimiento</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>29-May-26</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr"/>
+      <c r="K49" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-05-29 14:57:36)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,8 +28,12 @@
     <font>
       <color rgb="00000000"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00721C24"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -46,6 +50,11 @@
         <fgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8D7DA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -59,10 +68,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -428,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -634,7 +644,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>29-May-26</t>
+          <t>5-Jun-26</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
@@ -679,7 +689,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>29-May-26</t>
+          <t>5-Jun-26</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
@@ -769,7 +779,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>29-May-26</t>
+          <t>5-Jun-26</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr"/>
@@ -870,249 +880,233 @@
       <c r="K9" s="1" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Capacitar a personal nuevo ingreso Garcia Montoya Uriel Alejandro</t>
         </is>
       </c>
-      <c r="H10" s="2" t="n">
+      <c r="H10" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="J10" s="3" t="inlineStr"/>
+      <c r="K10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Capacitar a personal nuevo ingreso Alvarado Rojas Miguel Antonio</t>
         </is>
       </c>
-      <c r="H11" s="2" t="n">
+      <c r="H11" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="J11" s="3" t="inlineStr"/>
+      <c r="K11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Capacitar a personal nuevo ingreso Alvarado Aguilar Luis Alejandro</t>
         </is>
       </c>
-      <c r="H12" s="2" t="n">
+      <c r="H12" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="J12" s="3" t="inlineStr"/>
+      <c r="K12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Capacitar a personal nuevo ingreso XXXX</t>
         </is>
       </c>
-      <c r="H13" t="n">
+      <c r="H13" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
+      <c r="J13" s="3" t="inlineStr"/>
+      <c r="K13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Mejoras</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>📐 Doblez</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Cotizar Refacciones de maquinas Dobladoras</t>
         </is>
       </c>
-      <c r="H14" s="2" t="n">
+      <c r="H14" s="3" t="n">
         <v>45</v>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="I14" s="3" t="inlineStr">
         <is>
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="J14" s="3" t="inlineStr">
         <is>
           <t>12/May - Se mando Correo a Flex con Imágenes</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -1405,53 +1399,53 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Auto Asignado</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>👑 Direccion</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>Autorización compra de aspiradora para limpieza de Lijadora</t>
         </is>
       </c>
-      <c r="H21" s="2" t="n">
+      <c r="H21" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I21" s="3" t="inlineStr">
         <is>
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="J21" s="3" t="inlineStr">
         <is>
           <t>26/May - Requisición en SAI  21396 - REQ. HTA. PARTE 2JM</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr"/>
+      <c r="K21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -1544,53 +1538,53 @@
       <c r="K23" s="1" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>12-May-26</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>👑 Direccion</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>Autorización de Matriz Dobladora 85x85x3200</t>
         </is>
       </c>
-      <c r="H24" s="2" t="n">
+      <c r="H24" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="I24" s="3" t="inlineStr">
         <is>
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="J24" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">26/May - Requisición Aun no se tiene autorización 21485 - HERRAMENTAL DOBLEZ </t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr"/>
+      <c r="K24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -1638,57 +1632,53 @@
       <c r="K25" s="1" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
+      <c r="A26" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>12-May-26</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F26" s="3" t="inlineStr">
         <is>
           <t>👑 Direccion</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>Autorización de Escritorios y Sillas</t>
         </is>
       </c>
-      <c r="H26" s="2" t="n">
+      <c r="H26" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="I26" s="3" t="inlineStr">
         <is>
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="J26" s="3" t="inlineStr">
         <is>
           <t>28/May - Se a reenviado las Requisiciones al Ing. Alfredo para autorización 21348-21092</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -1875,49 +1865,49 @@
       <c r="K30" s="1" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" t="n">
+      <c r="A31" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>Acuerdos</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>18-May-26</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="3" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>Elaborar Procedimiento de Retrabajo de Barrenado puerta</t>
         </is>
       </c>
-      <c r="H31" t="n">
+      <c r="H31" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="I31" s="3" t="inlineStr">
         <is>
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
+      <c r="J31" s="3" t="inlineStr"/>
+      <c r="K31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -2436,11 +2426,7 @@
           <t>28/May - Hable con Cesar Campos (Ya llego a Monclova la van a mandar por paqueteria).</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2489,11 +2475,7 @@
           <t>28/May - Ajustando con el Organigrama oficial la actividad es separar al personal.</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2590,53 +2572,53 @@
       <c r="K45" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n">
+      <c r="A46" s="3" t="n">
         <v>45</v>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B46" s="3" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="C46" s="3" t="inlineStr">
         <is>
           <t>28-May-26</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
         <is>
           <t>Luis Quintana</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F46" s="3" t="inlineStr">
         <is>
           <t>🚚 Embarquez</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G46" s="3" t="inlineStr">
         <is>
           <t>26/May  - Comenzar el proceso de empaquetado del Material en DIAGONAL 1600 piezas</t>
         </is>
       </c>
-      <c r="H46" s="2" t="n">
+      <c r="H46" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="I46" s="2" t="inlineStr">
+      <c r="I46" s="3" t="inlineStr">
         <is>
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr">
+      <c r="J46" s="3" t="inlineStr">
         <is>
           <t>28/May - 26 Tarimas Preparadas Apro 35% avance  1 Dia despues</t>
         </is>
       </c>
-      <c r="K46" s="2" t="inlineStr"/>
+      <c r="K46" s="3" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2729,49 +2711,143 @@
       <c r="K48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n">
+      <c r="A49" s="3" t="n">
         <v>48</v>
       </c>
-      <c r="B49" s="2" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="C49" s="3" t="inlineStr">
         <is>
           <t>28-May-26</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
         <is>
           <t>Rodolfo Ferndez M</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr">
+      <c r="F49" s="3" t="inlineStr">
         <is>
           <t>⚙️ Ingenieria</t>
         </is>
       </c>
-      <c r="G49" s="2" t="inlineStr">
+      <c r="G49" s="3" t="inlineStr">
         <is>
           <t>Hacer 10 planos con las correcciones solicitadas por departamento de Calidad para estresar procedimiento</t>
         </is>
       </c>
-      <c r="H49" s="2" t="n">
+      <c r="H49" s="3" t="n">
         <v>90</v>
       </c>
-      <c r="I49" s="2" t="inlineStr">
+      <c r="I49" s="3" t="inlineStr">
         <is>
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J49" s="2" t="inlineStr"/>
-      <c r="K49" s="2" t="inlineStr"/>
+      <c r="J49" s="3" t="inlineStr"/>
+      <c r="K49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Mejoras</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>28-May-26</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Bryan Flores</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>👑 Direccion</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Limpieza de Terreno lateral cercado Planta Diagonal</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>12-Jun-26</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>27/May - Se hacen alguna Actividades de Limpieza ver evidencia carpeta MCE049</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Programa de Actividades</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>28-May-26</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Bryan Flores</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>✂️ Corte</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Corte de Placas de Tranformadores - Karime OT interna Sigrama 3 Placas</t>
+        </is>
+      </c>
+      <c r="H51" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>02-Jun-26</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-05-29 15:52:43)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -880,233 +880,233 @@
       <c r="K9" s="1" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n">
+      <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Capacitar a personal nuevo ingreso Garcia Montoya Uriel Alejandro</t>
         </is>
       </c>
-      <c r="H10" s="3" t="n">
+      <c r="H10" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>29-May-26</t>
-        </is>
-      </c>
-      <c r="J10" s="3" t="inlineStr"/>
-      <c r="K10" s="3" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>5-Jun-26</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Capacitar a personal nuevo ingreso Alvarado Rojas Miguel Antonio</t>
         </is>
       </c>
-      <c r="H11" s="3" t="n">
+      <c r="H11" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>29-May-26</t>
-        </is>
-      </c>
-      <c r="J11" s="3" t="inlineStr"/>
-      <c r="K11" s="3" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>5-Jun-26</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n">
+      <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Capacitar a personal nuevo ingreso Alvarado Aguilar Luis Alejandro</t>
         </is>
       </c>
-      <c r="H12" s="3" t="n">
+      <c r="H12" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>29-May-26</t>
-        </is>
-      </c>
-      <c r="J12" s="3" t="inlineStr"/>
-      <c r="K12" s="3" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>5-Jun-26</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n">
+      <c r="A13" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Capacitar a personal nuevo ingreso XXXX</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="n">
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Capacitar a personal nuevo ingreso David Alejandro Hernandez Rod</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
         <v>0</v>
       </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>29-May-26</t>
-        </is>
-      </c>
-      <c r="J13" s="3" t="inlineStr"/>
-      <c r="K13" s="3" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>5-Jun-26</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="n">
+      <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Mejoras</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>📐 Doblez</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Cotizar Refacciones de maquinas Dobladoras</t>
         </is>
       </c>
-      <c r="H14" s="3" t="n">
+      <c r="H14" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>29-May-26</t>
-        </is>
-      </c>
-      <c r="J14" s="3" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>5-Jun-26</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>12/May - Se mando Correo a Flex con Imágenes</t>
         </is>
       </c>
-      <c r="K14" s="3" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -1399,53 +1399,53 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n">
+      <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Auto Asignado</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>👑 Direccion</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>Autorización compra de aspiradora para limpieza de Lijadora</t>
         </is>
       </c>
-      <c r="H21" s="3" t="n">
+      <c r="H21" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>29-May-26</t>
-        </is>
-      </c>
-      <c r="J21" s="3" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>27-Jun-26</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
         <is>
           <t>26/May - Requisición en SAI  21396 - REQ. HTA. PARTE 2JM</t>
         </is>
       </c>
-      <c r="K21" s="3" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -1538,53 +1538,53 @@
       <c r="K23" s="1" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="n">
+      <c r="A24" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>12-May-26</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>👑 Direccion</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>Autorización de Matriz Dobladora 85x85x3200</t>
         </is>
       </c>
-      <c r="H24" s="3" t="n">
+      <c r="H24" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>29-May-26</t>
-        </is>
-      </c>
-      <c r="J24" s="3" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>27-Jun-26</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">26/May - Requisición Aun no se tiene autorización 21485 - HERRAMENTAL DOBLEZ </t>
         </is>
       </c>
-      <c r="K24" s="3" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -1865,49 +1865,49 @@
       <c r="K30" s="1" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="n">
+      <c r="A31" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>Acuerdos</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>18-May-26</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>Elaborar Procedimiento de Retrabajo de Barrenado puerta</t>
         </is>
       </c>
-      <c r="H31" s="3" t="n">
+      <c r="H31" t="n">
         <v>0</v>
       </c>
-      <c r="I31" s="3" t="inlineStr">
-        <is>
-          <t>29-May-26</t>
-        </is>
-      </c>
-      <c r="J31" s="3" t="inlineStr"/>
-      <c r="K31" s="3" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>5-Jun-26</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -2241,53 +2241,53 @@
       <c r="K38" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" t="n">
+      <c r="A39" s="1" t="n">
         <v>38</v>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="1" t="inlineStr">
         <is>
           <t>26-May-26</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="1" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E39" s="1" t="inlineStr">
         <is>
           <t>Luis Quintana</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F39" s="1" t="inlineStr">
         <is>
           <t>🚚 Embarquez</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="G39" s="1" t="inlineStr">
         <is>
           <t>Presentar a Cruz y Bryan en planta RIO Area de Compras</t>
         </is>
       </c>
-      <c r="H39" t="n">
-        <v>90</v>
-      </c>
-      <c r="I39" t="inlineStr">
+      <c r="H39" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I39" s="1" t="inlineStr">
         <is>
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="J39" s="1" t="inlineStr">
         <is>
           <t>26/Mayo - Presento a Bryan (No se pueden ir los 3 al mismo tiempo). Se programara visita cruz despues..!!!</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr"/>
+      <c r="K39" s="1" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -2572,53 +2572,53 @@
       <c r="K45" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="3" t="n">
+      <c r="A46" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="B46" s="3" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C46" s="3" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>28-May-26</t>
         </is>
       </c>
-      <c r="D46" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E46" s="3" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>Luis Quintana</t>
         </is>
       </c>
-      <c r="F46" s="3" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>🚚 Embarquez</t>
         </is>
       </c>
-      <c r="G46" s="3" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>26/May  - Comenzar el proceso de empaquetado del Material en DIAGONAL 1600 piezas</t>
         </is>
       </c>
-      <c r="H46" s="3" t="n">
+      <c r="H46" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="I46" s="3" t="inlineStr">
-        <is>
-          <t>29-May-26</t>
-        </is>
-      </c>
-      <c r="J46" s="3" t="inlineStr">
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>05-Jun-26</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
         <is>
           <t>28/May - 26 Tarimas Preparadas Apro 35% avance  1 Dia despues</t>
         </is>
       </c>
-      <c r="K46" s="3" t="inlineStr"/>
+      <c r="K46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2711,49 +2711,49 @@
       <c r="K48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="3" t="n">
+      <c r="A49" s="1" t="n">
         <v>48</v>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B49" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr">
+      <c r="C49" s="1" t="inlineStr">
         <is>
           <t>28-May-26</t>
         </is>
       </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="inlineStr">
+      <c r="D49" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E49" s="1" t="inlineStr">
         <is>
           <t>Rodolfo Ferndez M</t>
         </is>
       </c>
-      <c r="F49" s="3" t="inlineStr">
+      <c r="F49" s="1" t="inlineStr">
         <is>
           <t>⚙️ Ingenieria</t>
         </is>
       </c>
-      <c r="G49" s="3" t="inlineStr">
+      <c r="G49" s="1" t="inlineStr">
         <is>
           <t>Hacer 10 planos con las correcciones solicitadas por departamento de Calidad para estresar procedimiento</t>
         </is>
       </c>
-      <c r="H49" s="3" t="n">
-        <v>90</v>
-      </c>
-      <c r="I49" s="3" t="inlineStr">
+      <c r="H49" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I49" s="1" t="inlineStr">
         <is>
           <t>29-May-26</t>
         </is>
       </c>
-      <c r="J49" s="3" t="inlineStr"/>
-      <c r="K49" s="3" t="inlineStr"/>
+      <c r="J49" s="1" t="inlineStr"/>
+      <c r="K49" s="1" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-06-02 17:47:27)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K51"/>
+  <dimension ref="A1:K52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -606,94 +606,94 @@
       <c r="K3" s="1" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="1" t="inlineStr">
         <is>
           <t>Capacitar a personal nuevo ingreso Flores Campa Marvin Manuel</t>
         </is>
       </c>
-      <c r="H4" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="H4" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I4" s="1" t="inlineStr">
         <is>
           <t>5-Jun-26</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
+      <c r="J4" s="1" t="inlineStr"/>
+      <c r="K4" s="1" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="1" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="1" t="inlineStr">
         <is>
           <t>Capacitar a personal nuevo ingreso Campos Martinez Jesus Manuel</t>
         </is>
       </c>
-      <c r="H5" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="H5" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I5" s="1" t="inlineStr">
         <is>
           <t>5-Jun-26</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
+      <c r="J5" s="1" t="inlineStr"/>
+      <c r="K5" s="1" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -741,49 +741,49 @@
       <c r="K6" s="1" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" s="1" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" s="1" t="inlineStr">
         <is>
           <t>Capacitar a personal nuevo ingreso Alejandro Hernandez Perez</t>
         </is>
       </c>
-      <c r="H7" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="H7" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I7" s="1" t="inlineStr">
         <is>
           <t>5-Jun-26</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr"/>
+      <c r="J7" s="1" t="inlineStr"/>
+      <c r="K7" s="1" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -1632,53 +1632,53 @@
       <c r="K25" s="1" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="n">
+      <c r="A26" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>12-May-26</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F26" s="3" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>👑 Direccion</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>Autorización de Escritorios y Sillas</t>
         </is>
       </c>
-      <c r="H26" s="3" t="n">
+      <c r="H26" t="n">
         <v>30</v>
       </c>
-      <c r="I26" s="3" t="inlineStr">
-        <is>
-          <t>29-May-26</t>
-        </is>
-      </c>
-      <c r="J26" s="3" t="inlineStr">
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>31-Jun-26</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
         <is>
           <t>28/May - Se a reenviado las Requisiciones al Ing. Alfredo para autorización 21348-21092</t>
         </is>
       </c>
-      <c r="K26" s="3" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -2478,49 +2478,49 @@
       <c r="K43" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" t="n">
+      <c r="A44" s="1" t="n">
         <v>43</v>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="1" t="inlineStr">
         <is>
           <t>Procesos</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="1" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
+      <c r="D44" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E44" s="1" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F44" s="1" t="inlineStr">
         <is>
           <t>✂️ Corte</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="G44" s="1" t="inlineStr">
         <is>
           <t>Elaborar Procedimiento de Manufactura de Corte Laser.</t>
         </is>
       </c>
-      <c r="H44" t="n">
-        <v>0</v>
-      </c>
-      <c r="I44" t="inlineStr">
+      <c r="H44" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I44" s="1" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
+      <c r="J44" s="1" t="inlineStr"/>
+      <c r="K44" s="1" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2756,98 +2756,143 @@
       <c r="K49" s="1" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
+      <c r="A50" s="1" t="n">
         <v>49</v>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B50" s="1" t="inlineStr">
         <is>
           <t>Mejoras</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
+      <c r="C50" s="1" t="inlineStr">
         <is>
           <t>28-May-26</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="D50" s="1" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="E50" s="1" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="F50" s="1" t="inlineStr">
         <is>
           <t>👑 Direccion</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr">
+      <c r="G50" s="1" t="inlineStr">
         <is>
           <t>Limpieza de Terreno lateral cercado Planta Diagonal</t>
         </is>
       </c>
-      <c r="H50" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="I50" s="2" t="inlineStr">
+      <c r="H50" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I50" s="1" t="inlineStr">
         <is>
           <t>12-Jun-26</t>
         </is>
       </c>
-      <c r="J50" s="2" t="inlineStr">
+      <c r="J50" s="1" t="inlineStr">
         <is>
           <t>27/May - Se hacen alguna Actividades de Limpieza ver evidencia carpeta MCE049</t>
         </is>
       </c>
-      <c r="K50" s="2" t="inlineStr"/>
+      <c r="K50" s="1" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" t="n">
+      <c r="A51" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="1" t="inlineStr">
         <is>
           <t>28-May-26</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
+      <c r="D51" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E51" s="1" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="F51" s="1" t="inlineStr">
         <is>
           <t>✂️ Corte</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr">
+      <c r="G51" s="1" t="inlineStr">
         <is>
           <t>Corte de Placas de Tranformadores - Karime OT interna Sigrama 3 Placas</t>
         </is>
       </c>
-      <c r="H51" t="n">
+      <c r="H51" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I51" s="1" t="inlineStr">
+        <is>
+          <t>02-Jun-26</t>
+        </is>
+      </c>
+      <c r="J51" s="1" t="inlineStr"/>
+      <c r="K51" s="1" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Dirección</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>02-Jun-26</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>Urgente</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>🎨 Pintura</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>inventario retrabajo Galvatec</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I51" t="inlineStr">
+      <c r="I52" s="3" t="inlineStr">
         <is>
           <t>02-Jun-26</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
+      <c r="J52" s="3" t="inlineStr"/>
+      <c r="K52" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-06-03 14:27:57)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -880,184 +880,200 @@
       <c r="K9" s="1" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="1" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" s="1" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" s="1" t="inlineStr">
         <is>
           <t>Capacitar a personal nuevo ingreso Garcia Montoya Uriel Alejandro</t>
         </is>
       </c>
-      <c r="H10" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="H10" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I10" s="1" t="inlineStr">
         <is>
           <t>5-Jun-26</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr"/>
+      <c r="J10" s="1" t="inlineStr"/>
+      <c r="K10" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F11" s="1" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" s="1" t="inlineStr">
         <is>
           <t>Capacitar a personal nuevo ingreso Alvarado Rojas Miguel Antonio</t>
         </is>
       </c>
-      <c r="H11" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="H11" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I11" s="1" t="inlineStr">
         <is>
           <t>5-Jun-26</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="inlineStr"/>
+      <c r="J11" s="1" t="inlineStr"/>
+      <c r="K11" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="1" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F12" s="1" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" s="1" t="inlineStr">
         <is>
           <t>Capacitar a personal nuevo ingreso Alvarado Aguilar Luis Alejandro</t>
         </is>
       </c>
-      <c r="H12" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="H12" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I12" s="1" t="inlineStr">
         <is>
           <t>5-Jun-26</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr"/>
+      <c r="J12" s="1" t="inlineStr"/>
+      <c r="K12" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" s="1" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" s="1" t="inlineStr">
         <is>
           <t>Capacitar a personal nuevo ingreso David Alejandro Hernandez Rod</t>
         </is>
       </c>
-      <c r="H13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" t="inlineStr">
+      <c r="H13" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I13" s="1" t="inlineStr">
         <is>
           <t>5-Jun-26</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
+      <c r="J13" s="1" t="inlineStr"/>
+      <c r="K13" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1865,49 +1881,53 @@
       <c r="K30" s="1" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" t="n">
+      <c r="A31" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>Acuerdos</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>18-May-26</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>Elaborar Procedimiento de Retrabajo de Barrenado puerta</t>
         </is>
       </c>
-      <c r="H31" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" t="inlineStr">
+      <c r="H31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>5-Jun-26</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -2147,49 +2167,53 @@
       <c r="K36" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" t="n">
+      <c r="A37" s="1" t="n">
         <v>36</v>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="1" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
+      <c r="D37" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E37" s="1" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F37" s="1" t="inlineStr">
         <is>
           <t>✂️ Corte</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G37" s="1" t="inlineStr">
         <is>
           <t>Fabricar mesas para Tarimas con material reciclado, Altura ergonomica</t>
         </is>
       </c>
-      <c r="H37" t="n">
-        <v>0</v>
-      </c>
-      <c r="I37" t="inlineStr">
+      <c r="H37" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I37" s="1" t="inlineStr">
         <is>
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
+      <c r="J37" s="1" t="inlineStr"/>
+      <c r="K37" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2429,53 +2453,57 @@
       <c r="K42" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" t="n">
+      <c r="A43" s="1" t="n">
         <v>42</v>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="1" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
+      <c r="D43" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E43" s="1" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F43" s="1" t="inlineStr">
         <is>
           <t>✂️ Corte</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="G43" s="1" t="inlineStr">
         <is>
           <t>Hacer Nuevo Organigrama de Personal</t>
         </is>
       </c>
-      <c r="H43" t="n">
-        <v>70</v>
-      </c>
-      <c r="I43" t="inlineStr">
+      <c r="H43" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I43" s="1" t="inlineStr">
         <is>
           <t>2026-06-05</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="J43" s="1" t="inlineStr">
         <is>
           <t>28/May - Ajustando con el Organigrama oficial la actividad es separar al personal.</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr"/>
+      <c r="K43" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-06-03 14:30:18)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K52"/>
+  <dimension ref="A1:K53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2922,6 +2922,51 @@
       <c r="J52" s="3" t="inlineStr"/>
       <c r="K52" s="3" t="inlineStr"/>
     </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Mejoras</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>03-Jun-26</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Cruz Carreon</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>📐 Doblez</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Fabricar y ensamblar 2 Bases para Aires</t>
+        </is>
+      </c>
+      <c r="H53" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>09-Jun-26</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-06-03 14:40:05)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K53"/>
+  <dimension ref="A1:K57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2967,6 +2967,186 @@
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr"/>
     </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Mejoras</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>03-Jun-26</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Cruz Carreon</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>📐 Doblez</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Hacer requisición de Grasa para maquinas Dobladoras (Cremayeras)</t>
+        </is>
+      </c>
+      <c r="H54" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>05-Jun-26</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Procesos</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>03-Jun-26</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Cruz Carreon</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>📐 Doblez</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Elaborar Procedimiento del Area de Doblez (Primera Parte)</t>
+        </is>
+      </c>
+      <c r="H55" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>05-Jun-26</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Procesos</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>03-Jun-26</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Cruz Carreon</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>📐 Doblez</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Formato de Registro Diario de Doblez.</t>
+        </is>
+      </c>
+      <c r="H56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>05-Jun-26</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Mejoras</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>03-Jun-26</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Cruz Carreon</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>👑 Direccion</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Cerrar tapa de Insyalación Electrica Tablero de control Principal, Ver con Romo</t>
+        </is>
+      </c>
+      <c r="H57" t="n">
+        <v>0</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>05-Jun-26</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-06-03 15:24:10)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K57"/>
+  <dimension ref="A1:K69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2063,10 +2063,14 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>28/May - Pendiente modificar Requi.   Con Numeros Articulos nuevos</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr"/>
+          <t>03/Jun - Requisición Seguimiento</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2634,7 +2638,7 @@
         </is>
       </c>
       <c r="H46" s="2" t="n">
-        <v>35</v>
+        <v>70</v>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
@@ -2643,10 +2647,14 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>28/May - 26 Tarimas Preparadas Apro 35% avance  1 Dia despues</t>
-        </is>
-      </c>
-      <c r="K46" s="2" t="inlineStr"/>
+          <t>03/Jun - Avance 70%</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2878,49 +2886,57 @@
       <c r="K51" s="1" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="3" t="n">
+      <c r="A52" s="1" t="n">
         <v>51</v>
       </c>
-      <c r="B52" s="3" t="inlineStr">
+      <c r="B52" s="1" t="inlineStr">
         <is>
           <t>Dirección</t>
         </is>
       </c>
-      <c r="C52" s="3" t="inlineStr">
+      <c r="C52" s="1" t="inlineStr">
         <is>
           <t>02-Jun-26</t>
         </is>
       </c>
-      <c r="D52" s="3" t="inlineStr">
+      <c r="D52" s="1" t="inlineStr">
         <is>
           <t>Urgente</t>
         </is>
       </c>
-      <c r="E52" s="3" t="inlineStr">
+      <c r="E52" s="1" t="inlineStr">
         <is>
           <t>Luis Quintana</t>
         </is>
       </c>
-      <c r="F52" s="3" t="inlineStr">
+      <c r="F52" s="1" t="inlineStr">
         <is>
           <t>🎨 Pintura</t>
         </is>
       </c>
-      <c r="G52" s="3" t="inlineStr">
+      <c r="G52" s="1" t="inlineStr">
         <is>
           <t>inventario retrabajo Galvatec</t>
         </is>
       </c>
-      <c r="H52" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I52" s="3" t="inlineStr">
+      <c r="H52" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I52" s="1" t="inlineStr">
         <is>
           <t>02-Jun-26</t>
         </is>
       </c>
-      <c r="J52" s="3" t="inlineStr"/>
-      <c r="K52" s="3" t="inlineStr"/>
+      <c r="J52" s="1" t="inlineStr">
+        <is>
+          <t>03/Jun - Terminado Por enviar Reporte</t>
+        </is>
+      </c>
+      <c r="K52" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -3146,6 +3162,546 @@
       </c>
       <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Mejoras</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>03-Jun-26</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Cruz Carreon</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>⚙️ Ingenieria</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Instalar Interruptor de Extractor</t>
+        </is>
+      </c>
+      <c r="H58" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>12-Jun-26</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Programa de Actividades</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>03-Jun-26</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Urgente</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>🚚 Embarquez</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Elaborar Lista de Reposiciones para Proyecto Reno 6 Parcialidad 2.- Despues de Inventario</t>
+        </is>
+      </c>
+      <c r="H59" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>04-Jun-26</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Programa de Actividades</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>03-Jun-26</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Urgente</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>🚚 Embarquez</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Lista de Reposiciones Reno 6 Parcialodad 2</t>
+        </is>
+      </c>
+      <c r="H60" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>04-Jun-26</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Dirección</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>03-Jun-26</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>Urgente</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>Jesus Morales</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>👑 Direccion</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>Revvisión de Espacio para Almacenaje de Tarimas.</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>03-Jun-26</t>
+        </is>
+      </c>
+      <c r="J61" s="3" t="inlineStr"/>
+      <c r="K61" s="3" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Programa de Actividades</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>03-Jun-26</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Bryan Flores</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>✂️ Corte</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Identificar con Nuevo formato los datos de Atado de Materia Prima con sus atributos.</t>
+        </is>
+      </c>
+      <c r="H62" t="n">
+        <v>0</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>05-Jun-26</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Problema de Calidad</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>03-Jun-26</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Urgente</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Bryan Flores</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>✂️ Corte</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Poner Etiqueta ROJA de Material No conforme Lamina 12</t>
+        </is>
+      </c>
+      <c r="H63" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>04-Jun-26</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Problema de Calidad</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>03-Jun-26</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Urgente</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Bryan Flores</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>✂️ Corte</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Definir y Generar el WIP #1  Pos-laser</t>
+        </is>
+      </c>
+      <c r="H64" t="n">
+        <v>0</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>08-Jun-26</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Problema de Calidad</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>03-Jun-26</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Urgente</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Bryan Flores</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>✂️ Corte</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Impacto de Wip en Procedimiento</t>
+        </is>
+      </c>
+      <c r="H65" t="n">
+        <v>0</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>12-Jun-26</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Problema de Calidad</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>03-Jun-26</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Bryan Flores</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>✂️ Corte</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Archivos de Programa de Producción por Estación</t>
+        </is>
+      </c>
+      <c r="H66" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>12-Jun-26</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Programa de Actividades</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>03-Jun-26</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Rodolfo Ferndez M</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>⚙️ Ingenieria</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Revisión Con Cruz y Bryan del Procedimiento de Ingenieria</t>
+        </is>
+      </c>
+      <c r="H67" t="n">
+        <v>0</v>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>05-Jun-26</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Programa de Actividades</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>03-Jun-26</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Rodolfo Ferndez M</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>⚙️ Ingenieria</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Revisión Con Area de Calidad del Procedimiento </t>
+        </is>
+      </c>
+      <c r="H68" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>12-Jun-26</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Programa de Actividades</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>03-Jun-26</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Rodolfo Ferndez M</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>⚙️ Ingenieria</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Actualización de Planos Armando WOO Aprox. 70 Planos.</t>
+        </is>
+      </c>
+      <c r="H69" t="n">
+        <v>0</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>19-Jun-26</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-06-03 18:02:59)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -922,11 +922,7 @@
         </is>
       </c>
       <c r="J10" s="1" t="inlineStr"/>
-      <c r="K10" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K10" s="1" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -971,11 +967,7 @@
         </is>
       </c>
       <c r="J11" s="1" t="inlineStr"/>
-      <c r="K11" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K11" s="1" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -1020,11 +1012,7 @@
         </is>
       </c>
       <c r="J12" s="1" t="inlineStr"/>
-      <c r="K12" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K12" s="1" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -1069,11 +1057,7 @@
         </is>
       </c>
       <c r="J13" s="1" t="inlineStr"/>
-      <c r="K13" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K13" s="1" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1923,11 +1907,7 @@
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr"/>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -2066,11 +2046,7 @@
           <t>03/Jun - Requisición Seguimiento</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2213,11 +2189,7 @@
         </is>
       </c>
       <c r="J37" s="1" t="inlineStr"/>
-      <c r="K37" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K37" s="1" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2503,11 +2475,7 @@
           <t>28/May - Ajustando con el Organigrama oficial la actividad es separar al personal.</t>
         </is>
       </c>
-      <c r="K43" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K43" s="1" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
@@ -2650,11 +2618,7 @@
           <t>03/Jun - Avance 70%</t>
         </is>
       </c>
-      <c r="K46" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2932,11 +2896,7 @@
           <t>03/Jun - Terminado Por enviar Reporte</t>
         </is>
       </c>
-      <c r="K52" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K52" s="1" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-06-08 15:21:08)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -47,12 +47,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF3CD"/>
+        <fgColor rgb="00F8D7DA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8D7DA"/>
+        <fgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
   </fills>
@@ -71,8 +71,8 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1399,53 +1399,53 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Auto Asignado</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>👑 Direccion</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>Autorización compra de aspiradora para limpieza de Lijadora</t>
         </is>
       </c>
-      <c r="H21" s="2" t="n">
+      <c r="H21" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I21" s="3" t="inlineStr">
         <is>
           <t>27-Jun-26</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="J21" s="3" t="inlineStr">
         <is>
           <t>26/May - Requisición en SAI  21396 - REQ. HTA. PARTE 2JM</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr"/>
+      <c r="K21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -1538,53 +1538,53 @@
       <c r="K23" s="1" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>12-May-26</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>👑 Direccion</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>Autorización de Matriz Dobladora 85x85x3200</t>
         </is>
       </c>
-      <c r="H24" s="2" t="n">
+      <c r="H24" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="I24" s="3" t="inlineStr">
         <is>
           <t>27-Jun-26</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="J24" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">26/May - Requisición Aun no se tiene autorización 21485 - HERRAMENTAL DOBLEZ </t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr"/>
+      <c r="K24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -1726,49 +1726,53 @@
       <c r="K27" s="1" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="n">
+      <c r="A28" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>12-May-26</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>✂️ Corte</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>Diseño de Carro de Herramental Doblez</t>
         </is>
       </c>
-      <c r="H28" t="n">
-        <v>0</v>
-      </c>
-      <c r="I28" t="inlineStr">
+      <c r="H28" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>5-Jun-26</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -1865,49 +1869,53 @@
       <c r="K30" s="1" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
+      <c r="A31" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B31" s="1" t="inlineStr">
         <is>
           <t>Acuerdos</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C31" s="1" t="inlineStr">
         <is>
           <t>18-May-26</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D31" s="1" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E31" s="1" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="F31" s="1" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="G31" s="1" t="inlineStr">
         <is>
           <t>Elaborar Procedimiento de Retrabajo de Barrenado puerta</t>
         </is>
       </c>
-      <c r="H31" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="I31" s="2" t="inlineStr">
+      <c r="H31" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I31" s="1" t="inlineStr">
         <is>
           <t>5-Jun-26</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr"/>
-      <c r="K31" s="2" t="inlineStr"/>
+      <c r="J31" s="1" t="inlineStr"/>
+      <c r="K31" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -2621,49 +2629,49 @@
       <c r="K46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" t="n">
+      <c r="A47" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>Dirección</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>28-May-26</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>Luis Quintana</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>📦 Almacen</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t>Reubicar los racks a la pared bajo el Extractor.</t>
         </is>
       </c>
-      <c r="H47" t="n">
+      <c r="H47" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="I47" s="2" t="inlineStr">
         <is>
           <t>05-Jun-26</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr"/>
+      <c r="K47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -2944,184 +2952,196 @@
       <c r="K53" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" t="n">
+      <c r="A54" s="2" t="n">
         <v>53</v>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>Mejoras</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>📐 Doblez</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr">
+      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>Hacer requisición de Grasa para maquinas Dobladoras (Cremayeras)</t>
         </is>
       </c>
-      <c r="H54" t="n">
+      <c r="H54" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I54" t="inlineStr">
+      <c r="I54" s="2" t="inlineStr">
         <is>
           <t>05-Jun-26</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
+      <c r="J54" s="2" t="inlineStr"/>
+      <c r="K54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" t="n">
+      <c r="A55" s="1" t="n">
         <v>54</v>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B55" s="1" t="inlineStr">
         <is>
           <t>Procesos</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="1" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
+      <c r="D55" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E55" s="1" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr">
+      <c r="F55" s="1" t="inlineStr">
         <is>
           <t>📐 Doblez</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr">
+      <c r="G55" s="1" t="inlineStr">
         <is>
           <t>Elaborar Procedimiento del Area de Doblez (Primera Parte)</t>
         </is>
       </c>
-      <c r="H55" t="n">
-        <v>0</v>
-      </c>
-      <c r="I55" t="inlineStr">
+      <c r="H55" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I55" s="1" t="inlineStr">
         <is>
           <t>05-Jun-26</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
+      <c r="J55" s="1" t="inlineStr"/>
+      <c r="K55" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" t="n">
+      <c r="A56" s="1" t="n">
         <v>55</v>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B56" s="1" t="inlineStr">
         <is>
           <t>Procesos</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C56" s="1" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
+      <c r="D56" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E56" s="1" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="F56" s="1" t="inlineStr">
         <is>
           <t>📐 Doblez</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr">
+      <c r="G56" s="1" t="inlineStr">
         <is>
           <t>Formato de Registro Diario de Doblez.</t>
         </is>
       </c>
-      <c r="H56" t="n">
-        <v>0</v>
-      </c>
-      <c r="I56" t="inlineStr">
+      <c r="H56" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I56" s="1" t="inlineStr">
         <is>
           <t>05-Jun-26</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
+      <c r="J56" s="1" t="inlineStr"/>
+      <c r="K56" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="57">
-      <c r="A57" t="n">
+      <c r="A57" s="1" t="n">
         <v>56</v>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B57" s="1" t="inlineStr">
         <is>
           <t>Mejoras</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C57" s="1" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D57" s="1" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="E57" s="1" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
+      <c r="F57" s="1" t="inlineStr">
         <is>
           <t>👑 Direccion</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr">
+      <c r="G57" s="1" t="inlineStr">
         <is>
           <t>Cerrar tapa de Insyalación Electrica Tablero de control Principal, Ver con Romo</t>
         </is>
       </c>
-      <c r="H57" t="n">
-        <v>0</v>
-      </c>
-      <c r="I57" t="inlineStr">
+      <c r="H57" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I57" s="1" t="inlineStr">
         <is>
           <t>05-Jun-26</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
+      <c r="J57" s="1" t="inlineStr"/>
+      <c r="K57" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -3169,274 +3189,274 @@
       <c r="K58" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" t="n">
+      <c r="A59" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>Urgente</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>Luis Quintana</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr">
+      <c r="F59" s="2" t="inlineStr">
         <is>
           <t>🚚 Embarquez</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr">
+      <c r="G59" s="2" t="inlineStr">
         <is>
           <t>Elaborar Lista de Reposiciones para Proyecto Reno 6 Parcialidad 2.- Despues de Inventario</t>
         </is>
       </c>
-      <c r="H59" t="n">
+      <c r="H59" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I59" t="inlineStr">
+      <c r="I59" s="2" t="inlineStr">
         <is>
           <t>04-Jun-26</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
+      <c r="J59" s="2" t="inlineStr"/>
+      <c r="K59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" t="n">
+      <c r="A60" s="2" t="n">
         <v>59</v>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>Urgente</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>Luis Quintana</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr">
+      <c r="F60" s="2" t="inlineStr">
         <is>
           <t>🚚 Embarquez</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr">
+      <c r="G60" s="2" t="inlineStr">
         <is>
           <t>Lista de Reposiciones Reno 6 Parcialodad 2</t>
         </is>
       </c>
-      <c r="H60" t="n">
+      <c r="H60" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I60" t="inlineStr">
+      <c r="I60" s="2" t="inlineStr">
         <is>
           <t>04-Jun-26</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr"/>
+      <c r="K60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="3" t="n">
+      <c r="A61" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="B61" s="3" t="inlineStr">
+      <c r="B61" s="2" t="inlineStr">
         <is>
           <t>Dirección</t>
         </is>
       </c>
-      <c r="C61" s="3" t="inlineStr">
+      <c r="C61" s="2" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D61" s="3" t="inlineStr">
+      <c r="D61" s="2" t="inlineStr">
         <is>
           <t>Urgente</t>
         </is>
       </c>
-      <c r="E61" s="3" t="inlineStr">
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F61" s="3" t="inlineStr">
+      <c r="F61" s="2" t="inlineStr">
         <is>
           <t>👑 Direccion</t>
         </is>
       </c>
-      <c r="G61" s="3" t="inlineStr">
+      <c r="G61" s="2" t="inlineStr">
         <is>
           <t>Revvisión de Espacio para Almacenaje de Tarimas.</t>
         </is>
       </c>
-      <c r="H61" s="3" t="n">
+      <c r="H61" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I61" s="3" t="inlineStr">
+      <c r="I61" s="2" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="J61" s="3" t="inlineStr"/>
-      <c r="K61" s="3" t="inlineStr"/>
+      <c r="J61" s="2" t="inlineStr"/>
+      <c r="K61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" t="n">
+      <c r="A62" s="1" t="n">
         <v>61</v>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B62" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C62" s="1" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
+      <c r="D62" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E62" s="1" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
+      <c r="F62" s="1" t="inlineStr">
         <is>
           <t>✂️ Corte</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr">
+      <c r="G62" s="1" t="inlineStr">
         <is>
           <t>Identificar con Nuevo formato los datos de Atado de Materia Prima con sus atributos.</t>
         </is>
       </c>
-      <c r="H62" t="n">
+      <c r="H62" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I62" s="1" t="inlineStr">
+        <is>
+          <t>05-Jun-26</t>
+        </is>
+      </c>
+      <c r="J62" s="1" t="inlineStr"/>
+      <c r="K62" s="1" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="1" t="inlineStr">
+        <is>
+          <t>Problema de Calidad</t>
+        </is>
+      </c>
+      <c r="C63" s="1" t="inlineStr">
+        <is>
+          <t>03-Jun-26</t>
+        </is>
+      </c>
+      <c r="D63" s="1" t="inlineStr">
+        <is>
+          <t>Urgente</t>
+        </is>
+      </c>
+      <c r="E63" s="1" t="inlineStr">
+        <is>
+          <t>Bryan Flores</t>
+        </is>
+      </c>
+      <c r="F63" s="1" t="inlineStr">
+        <is>
+          <t>✂️ Corte</t>
+        </is>
+      </c>
+      <c r="G63" s="1" t="inlineStr">
+        <is>
+          <t>Poner Etiqueta ROJA de Material No conforme Lamina 12</t>
+        </is>
+      </c>
+      <c r="H63" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I63" s="1" t="inlineStr">
+        <is>
+          <t>04-Jun-26</t>
+        </is>
+      </c>
+      <c r="J63" s="1" t="inlineStr"/>
+      <c r="K63" s="1" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Problema de Calidad</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>03-Jun-26</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Urgente</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Bryan Flores</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>✂️ Corte</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Definir y Generar el WIP #1  Pos-laser</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>05-Jun-26</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" t="n">
-        <v>62</v>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Problema de Calidad</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>03-Jun-26</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>Urgente</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Bryan Flores</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>✂️ Corte</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>Poner Etiqueta ROJA de Material No conforme Lamina 12</t>
-        </is>
-      </c>
-      <c r="H63" t="n">
-        <v>0</v>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>04-Jun-26</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" t="n">
-        <v>63</v>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>Problema de Calidad</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>03-Jun-26</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>Urgente</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Bryan Flores</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>✂️ Corte</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>Definir y Generar el WIP #1  Pos-laser</t>
-        </is>
-      </c>
-      <c r="H64" t="n">
-        <v>0</v>
-      </c>
-      <c r="I64" t="inlineStr">
+      <c r="I64" s="2" t="inlineStr">
         <is>
           <t>08-Jun-26</t>
         </is>
       </c>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
+      <c r="J64" s="2" t="inlineStr"/>
+      <c r="K64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -3529,49 +3549,49 @@
       <c r="K66" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" t="n">
+      <c r="A67" s="2" t="n">
         <v>66</v>
       </c>
-      <c r="B67" t="inlineStr">
+      <c r="B67" s="2" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="C67" s="2" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
         <is>
           <t>Rodolfo Ferndez M</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr">
+      <c r="F67" s="2" t="inlineStr">
         <is>
           <t>⚙️ Ingenieria</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr">
+      <c r="G67" s="2" t="inlineStr">
         <is>
           <t>Revisión Con Cruz y Bryan del Procedimiento de Ingenieria</t>
         </is>
       </c>
-      <c r="H67" t="n">
+      <c r="H67" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I67" t="inlineStr">
+      <c r="I67" s="2" t="inlineStr">
         <is>
           <t>05-Jun-26</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
+      <c r="J67" s="2" t="inlineStr"/>
+      <c r="K67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-06-08 16:15:49)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K69"/>
+  <dimension ref="A1:K70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1768,11 +1768,7 @@
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -1911,11 +1907,7 @@
         </is>
       </c>
       <c r="J31" s="1" t="inlineStr"/>
-      <c r="K31" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K31" s="1" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -3039,11 +3031,7 @@
         </is>
       </c>
       <c r="J55" s="1" t="inlineStr"/>
-      <c r="K55" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K55" s="1" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
@@ -3088,11 +3076,7 @@
         </is>
       </c>
       <c r="J56" s="1" t="inlineStr"/>
-      <c r="K56" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K56" s="1" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
@@ -3137,11 +3121,7 @@
         </is>
       </c>
       <c r="J57" s="1" t="inlineStr"/>
-      <c r="K57" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K57" s="1" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -3279,49 +3259,57 @@
       <c r="K60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n">
+      <c r="A61" s="1" t="n">
         <v>60</v>
       </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="B61" s="1" t="inlineStr">
         <is>
           <t>Dirección</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
+      <c r="C61" s="1" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="D61" s="1" t="inlineStr">
         <is>
           <t>Urgente</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="E61" s="1" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F61" s="2" t="inlineStr">
+      <c r="F61" s="1" t="inlineStr">
         <is>
           <t>👑 Direccion</t>
         </is>
       </c>
-      <c r="G61" s="2" t="inlineStr">
+      <c r="G61" s="1" t="inlineStr">
         <is>
           <t>Revvisión de Espacio para Almacenaje de Tarimas.</t>
         </is>
       </c>
-      <c r="H61" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I61" s="2" t="inlineStr">
+      <c r="H61" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I61" s="1" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="J61" s="2" t="inlineStr"/>
-      <c r="K61" s="2" t="inlineStr"/>
+      <c r="J61" s="1" t="inlineStr">
+        <is>
+          <t>03/Jun - Se decide hacer un Sistema para Empaque Solo este Alcance</t>
+        </is>
+      </c>
+      <c r="K61" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
@@ -3682,6 +3670,51 @@
       </c>
       <c r="J69" t="inlineStr"/>
       <c r="K69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Mejoras</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>08-Jun-26</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Jesus Morales</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>⚙️ Ingenieria</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Actualizar formato de Nombramiento de Archivos asi como Revisión de Objetivos del Procedimiento de Ingenieria Interno.</t>
+        </is>
+      </c>
+      <c r="H70" t="n">
+        <v>0</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>09-Jun-26</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-06-08 16:18:37)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -2899,49 +2899,53 @@
       <c r="K52" s="1" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" t="n">
+      <c r="A53" s="1" t="n">
         <v>52</v>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B53" s="1" t="inlineStr">
         <is>
           <t>Mejoras</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C53" s="1" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D53" s="1" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E53" s="1" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F53" s="1" t="inlineStr">
         <is>
           <t>📐 Doblez</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
+      <c r="G53" s="1" t="inlineStr">
         <is>
           <t>Fabricar y ensamblar 2 Bases para Aires</t>
         </is>
       </c>
-      <c r="H53" t="n">
-        <v>0</v>
-      </c>
-      <c r="I53" t="inlineStr">
+      <c r="H53" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I53" s="1" t="inlineStr">
         <is>
           <t>09-Jun-26</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
+      <c r="J53" s="1" t="inlineStr"/>
+      <c r="K53" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -3672,49 +3676,53 @@
       <c r="K69" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" t="n">
+      <c r="A70" s="1" t="n">
         <v>69</v>
       </c>
-      <c r="B70" t="inlineStr">
+      <c r="B70" s="1" t="inlineStr">
         <is>
           <t>Mejoras</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
+      <c r="C70" s="1" t="inlineStr">
         <is>
           <t>08-Jun-26</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
+      <c r="D70" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E70" s="1" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr">
+      <c r="F70" s="1" t="inlineStr">
         <is>
           <t>⚙️ Ingenieria</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr">
+      <c r="G70" s="1" t="inlineStr">
         <is>
           <t>Actualizar formato de Nombramiento de Archivos asi como Revisión de Objetivos del Procedimiento de Ingenieria Interno.</t>
         </is>
       </c>
-      <c r="H70" t="n">
-        <v>0</v>
-      </c>
-      <c r="I70" t="inlineStr">
+      <c r="H70" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I70" s="1" t="inlineStr">
         <is>
           <t>09-Jun-26</t>
         </is>
       </c>
-      <c r="J70" t="inlineStr"/>
-      <c r="K70" t="inlineStr"/>
+      <c r="J70" s="1" t="inlineStr"/>
+      <c r="K70" s="1" t="inlineStr">
+        <is>
+          <t>evidencias/MCE-069_evidencia_20260608_161744.jpg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-06-08 17:29:26)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K70"/>
+  <dimension ref="A1:K71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1768,7 +1768,11 @@
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -1907,7 +1911,11 @@
         </is>
       </c>
       <c r="J31" s="1" t="inlineStr"/>
-      <c r="K31" s="1" t="inlineStr"/>
+      <c r="K31" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -2899,53 +2907,49 @@
       <c r="K52" s="1" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
+      <c r="A53" t="n">
         <v>52</v>
       </c>
-      <c r="B53" s="1" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>Mejoras</t>
         </is>
       </c>
-      <c r="C53" s="1" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D53" s="1" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E53" s="1" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F53" s="1" t="inlineStr">
+      <c r="F53" t="inlineStr">
         <is>
           <t>📐 Doblez</t>
         </is>
       </c>
-      <c r="G53" s="1" t="inlineStr">
+      <c r="G53" t="inlineStr">
         <is>
           <t>Fabricar y ensamblar 2 Bases para Aires</t>
         </is>
       </c>
-      <c r="H53" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="I53" s="1" t="inlineStr">
+      <c r="H53" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" t="inlineStr">
         <is>
           <t>09-Jun-26</t>
         </is>
       </c>
-      <c r="J53" s="1" t="inlineStr"/>
-      <c r="K53" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -3035,7 +3039,11 @@
         </is>
       </c>
       <c r="J55" s="1" t="inlineStr"/>
-      <c r="K55" s="1" t="inlineStr"/>
+      <c r="K55" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
@@ -3080,7 +3088,11 @@
         </is>
       </c>
       <c r="J56" s="1" t="inlineStr"/>
-      <c r="K56" s="1" t="inlineStr"/>
+      <c r="K56" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
@@ -3125,7 +3137,11 @@
         </is>
       </c>
       <c r="J57" s="1" t="inlineStr"/>
-      <c r="K57" s="1" t="inlineStr"/>
+      <c r="K57" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -3263,57 +3279,49 @@
       <c r="K60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="n">
+      <c r="A61" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="B61" s="1" t="inlineStr">
+      <c r="B61" s="2" t="inlineStr">
         <is>
           <t>Dirección</t>
         </is>
       </c>
-      <c r="C61" s="1" t="inlineStr">
+      <c r="C61" s="2" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D61" s="1" t="inlineStr">
+      <c r="D61" s="2" t="inlineStr">
         <is>
           <t>Urgente</t>
         </is>
       </c>
-      <c r="E61" s="1" t="inlineStr">
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F61" s="1" t="inlineStr">
+      <c r="F61" s="2" t="inlineStr">
         <is>
           <t>👑 Direccion</t>
         </is>
       </c>
-      <c r="G61" s="1" t="inlineStr">
+      <c r="G61" s="2" t="inlineStr">
         <is>
           <t>Revvisión de Espacio para Almacenaje de Tarimas.</t>
         </is>
       </c>
-      <c r="H61" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="I61" s="1" t="inlineStr">
+      <c r="H61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="J61" s="1" t="inlineStr">
-        <is>
-          <t>03/Jun - Se decide hacer un Sistema para Empaque Solo este Alcance</t>
-        </is>
-      </c>
-      <c r="K61" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="J61" s="2" t="inlineStr"/>
+      <c r="K61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
@@ -3691,7 +3699,7 @@
       </c>
       <c r="D70" s="1" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="E70" s="1" t="inlineStr">
@@ -3701,12 +3709,12 @@
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>⚙️ Ingenieria</t>
+          <t>🚚 Embarquez</t>
         </is>
       </c>
       <c r="G70" s="1" t="inlineStr">
         <is>
-          <t>Actualizar formato de Nombramiento de Archivos asi como Revisión de Objetivos del Procedimiento de Ingenieria Interno.</t>
+          <t>Desarrollo de sistema de Embarquez</t>
         </is>
       </c>
       <c r="H70" s="1" t="n">
@@ -3714,15 +3722,60 @@
       </c>
       <c r="I70" s="1" t="inlineStr">
         <is>
-          <t>09-Jun-26</t>
+          <t>12-Jun-26</t>
         </is>
       </c>
       <c r="J70" s="1" t="inlineStr"/>
       <c r="K70" s="1" t="inlineStr">
         <is>
-          <t>evidencias/MCE-069_evidencia_20260608_161744.jpg</t>
-        </is>
-      </c>
+          <t>evidencias/MCE-069_evidencia_20260608_172743.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Acuerdos</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>08-Jun-26</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Jesus Morales</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>⚙️ Ingenieria</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Elaborar lista de Objetivos del Procedimiento de Ingenieria</t>
+        </is>
+      </c>
+      <c r="H71" t="n">
+        <v>0</v>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>09-Jun-26</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-06-08 19:07:33)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -1768,11 +1768,7 @@
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -1911,11 +1907,7 @@
         </is>
       </c>
       <c r="J31" s="1" t="inlineStr"/>
-      <c r="K31" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K31" s="1" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -2907,49 +2899,53 @@
       <c r="K52" s="1" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" t="n">
+      <c r="A53" s="1" t="n">
         <v>52</v>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B53" s="1" t="inlineStr">
         <is>
           <t>Mejoras</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C53" s="1" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D53" s="1" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E53" s="1" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F53" s="1" t="inlineStr">
         <is>
           <t>📐 Doblez</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
+      <c r="G53" s="1" t="inlineStr">
         <is>
           <t>Fabricar y ensamblar 2 Bases para Aires</t>
         </is>
       </c>
-      <c r="H53" t="n">
-        <v>0</v>
-      </c>
-      <c r="I53" t="inlineStr">
+      <c r="H53" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I53" s="1" t="inlineStr">
         <is>
           <t>09-Jun-26</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
+      <c r="J53" s="1" t="inlineStr"/>
+      <c r="K53" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -3039,11 +3035,7 @@
         </is>
       </c>
       <c r="J55" s="1" t="inlineStr"/>
-      <c r="K55" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K55" s="1" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
@@ -3088,11 +3080,7 @@
         </is>
       </c>
       <c r="J56" s="1" t="inlineStr"/>
-      <c r="K56" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K56" s="1" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
@@ -3137,11 +3125,7 @@
         </is>
       </c>
       <c r="J57" s="1" t="inlineStr"/>
-      <c r="K57" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K57" s="1" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -3279,49 +3263,57 @@
       <c r="K60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n">
+      <c r="A61" s="1" t="n">
         <v>60</v>
       </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="B61" s="1" t="inlineStr">
         <is>
           <t>Dirección</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
+      <c r="C61" s="1" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="D61" s="1" t="inlineStr">
         <is>
           <t>Urgente</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="E61" s="1" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F61" s="2" t="inlineStr">
+      <c r="F61" s="1" t="inlineStr">
         <is>
           <t>👑 Direccion</t>
         </is>
       </c>
-      <c r="G61" s="2" t="inlineStr">
+      <c r="G61" s="1" t="inlineStr">
         <is>
           <t>Revvisión de Espacio para Almacenaje de Tarimas.</t>
         </is>
       </c>
-      <c r="H61" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I61" s="2" t="inlineStr">
+      <c r="H61" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I61" s="1" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="J61" s="2" t="inlineStr"/>
-      <c r="K61" s="2" t="inlineStr"/>
+      <c r="J61" s="1" t="inlineStr">
+        <is>
+          <t>03/Jun - Se decide hacer un Sistema para Empaque Solo este Alcance</t>
+        </is>
+      </c>
+      <c r="K61" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
@@ -3699,7 +3691,7 @@
       </c>
       <c r="D70" s="1" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E70" s="1" t="inlineStr">
@@ -3709,12 +3701,12 @@
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>🚚 Embarquez</t>
+          <t>⚙️ Ingenieria</t>
         </is>
       </c>
       <c r="G70" s="1" t="inlineStr">
         <is>
-          <t>Desarrollo de sistema de Embarquez</t>
+          <t>Actualizar formato de Nombramiento de Archivos asi como Revisión de Objetivos del Procedimiento de Ingenieria Interno.</t>
         </is>
       </c>
       <c r="H70" s="1" t="n">
@@ -3722,60 +3714,60 @@
       </c>
       <c r="I70" s="1" t="inlineStr">
         <is>
-          <t>12-Jun-26</t>
+          <t>09-Jun-26</t>
         </is>
       </c>
       <c r="J70" s="1" t="inlineStr"/>
       <c r="K70" s="1" t="inlineStr">
         <is>
-          <t>evidencias/MCE-069_evidencia_20260608_172743.jpg</t>
+          <t>evidencias/MCE-069_evidencia_20260608_161744.jpg</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="n">
+      <c r="A71" s="1" t="n">
         <v>70</v>
       </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Acuerdos</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
+      <c r="B71" s="1" t="inlineStr">
+        <is>
+          <t>Programa de Actividades</t>
+        </is>
+      </c>
+      <c r="C71" s="1" t="inlineStr">
         <is>
           <t>08-Jun-26</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
+      <c r="D71" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E71" s="1" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>⚙️ Ingenieria</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>Elaborar lista de Objetivos del Procedimiento de Ingenieria</t>
-        </is>
-      </c>
-      <c r="H71" t="n">
-        <v>0</v>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>09-Jun-26</t>
-        </is>
-      </c>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
+      <c r="F71" s="1" t="inlineStr">
+        <is>
+          <t>🚚 Embarquez</t>
+        </is>
+      </c>
+      <c r="G71" s="1" t="inlineStr">
+        <is>
+          <t>Desarrollo de SISEMA DE EMBARQUES.</t>
+        </is>
+      </c>
+      <c r="H71" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I71" s="1" t="inlineStr">
+        <is>
+          <t>08-Jun-26</t>
+        </is>
+      </c>
+      <c r="J71" s="1" t="inlineStr"/>
+      <c r="K71" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-06-08 21:14:10)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K71"/>
+  <dimension ref="A1:K72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3769,6 +3769,51 @@
       <c r="J71" s="1" t="inlineStr"/>
       <c r="K71" s="1" t="inlineStr"/>
     </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Mejoras</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>08-Jun-26</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Jesus Morales</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>👥 Recursos Humanos</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Generar la Aplicación para revisar la PRENOMINA y que los lideres tomen acciones con Personal</t>
+        </is>
+      </c>
+      <c r="H72" t="n">
+        <v>0</v>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>12-Jun-26</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-06-08 22:07:14)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K72"/>
+  <dimension ref="A1:K73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2941,11 +2941,7 @@
         </is>
       </c>
       <c r="J53" s="1" t="inlineStr"/>
-      <c r="K53" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K53" s="1" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -3309,11 +3305,7 @@
           <t>03/Jun - Se decide hacer un Sistema para Empaque Solo este Alcance</t>
         </is>
       </c>
-      <c r="K61" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K61" s="1" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
@@ -3813,6 +3805,52 @@
       </c>
       <c r="J72" t="inlineStr"/>
       <c r="K72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Mejoras</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>08-Jun-26</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Jesus Morales</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>👑 Direccion</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Agregar un Reporte al MCE en la Dashboard
+</t>
+        </is>
+      </c>
+      <c r="H73" t="n">
+        <v>0</v>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>12-Jun-26</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-06-08 22:50:57)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -2380,53 +2380,57 @@
       <c r="K41" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" t="n">
+      <c r="A42" s="1" t="n">
         <v>41</v>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="1" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
+      <c r="D42" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E42" s="1" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F42" s="1" t="inlineStr">
         <is>
           <t>⚙️ Ingenieria</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="G42" s="1" t="inlineStr">
         <is>
           <t>Licencia PRONEST final</t>
         </is>
       </c>
-      <c r="H42" t="n">
-        <v>90</v>
-      </c>
-      <c r="I42" t="inlineStr">
+      <c r="H42" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I42" s="1" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="J42" s="1" t="inlineStr">
         <is>
           <t>28/May - Hable con Cesar Campos (Ya llego a Monclova la van a mandar por paqueteria).</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
+      <c r="K42" s="1" t="inlineStr">
+        <is>
+          <t>evidencias/MCE-041_evidencia_20260608_225041.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-06-08 22:59:51)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -2458,7 +2458,7 @@
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>✂️ Corte</t>
+          <t>📐 Doblez</t>
         </is>
       </c>
       <c r="G43" s="1" t="inlineStr">
@@ -3766,95 +3766,95 @@
       <c r="K71" s="1" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" t="n">
+      <c r="A72" s="1" t="n">
         <v>71</v>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B72" s="1" t="inlineStr">
         <is>
           <t>Mejoras</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C72" s="1" t="inlineStr">
         <is>
           <t>08-Jun-26</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
+      <c r="D72" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E72" s="1" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr">
+      <c r="F72" s="1" t="inlineStr">
         <is>
           <t>👥 Recursos Humanos</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr">
+      <c r="G72" s="1" t="inlineStr">
         <is>
           <t>Generar la Aplicación para revisar la PRENOMINA y que los lideres tomen acciones con Personal</t>
         </is>
       </c>
-      <c r="H72" t="n">
-        <v>0</v>
-      </c>
-      <c r="I72" t="inlineStr">
+      <c r="H72" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I72" s="1" t="inlineStr">
         <is>
           <t>12-Jun-26</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
+      <c r="J72" s="1" t="inlineStr"/>
+      <c r="K72" s="1" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" t="n">
+      <c r="A73" s="1" t="n">
         <v>72</v>
       </c>
-      <c r="B73" t="inlineStr">
+      <c r="B73" s="1" t="inlineStr">
         <is>
           <t>Mejoras</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="C73" s="1" t="inlineStr">
         <is>
           <t>08-Jun-26</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr">
+      <c r="D73" s="1" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr">
+      <c r="E73" s="1" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr">
+      <c r="F73" s="1" t="inlineStr">
         <is>
           <t>👑 Direccion</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr">
+      <c r="G73" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Agregar un Reporte al MCE en la Dashboard
 </t>
         </is>
       </c>
-      <c r="H73" t="n">
-        <v>0</v>
-      </c>
-      <c r="I73" t="inlineStr">
+      <c r="H73" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I73" s="1" t="inlineStr">
         <is>
           <t>12-Jun-26</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="inlineStr"/>
+      <c r="J73" s="1" t="inlineStr"/>
+      <c r="K73" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-06-08 23:53:29)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K73"/>
+  <dimension ref="A1:K74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1572,7 +1572,7 @@
         </is>
       </c>
       <c r="H24" s="3" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
@@ -1584,7 +1584,11 @@
           <t xml:space="preserve">26/May - Requisición Aun no se tiene autorización 21485 - HERRAMENTAL DOBLEZ </t>
         </is>
       </c>
-      <c r="K24" s="3" t="inlineStr"/>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -1666,7 +1670,7 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -1678,7 +1682,11 @@
           <t>28/May - Se a reenviado las Requisiciones al Ing. Alfredo para autorización 21348-21092</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -2083,7 +2091,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -2095,7 +2103,11 @@
           <t>28/May - Solicitud eviada al Ing. Alfredo de PC para Ing. Rodolfo.</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -3855,6 +3867,51 @@
       </c>
       <c r="J73" s="1" t="inlineStr"/>
       <c r="K73" s="1" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Programa de Actividades</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>08-Jun-26</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>🚚 Embarquez</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Generar Correo electronico de la Primera Remisión Generada en Programa de METALES.</t>
+        </is>
+      </c>
+      <c r="H74" t="n">
+        <v>0</v>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>12-Jun-26</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-06-09 17:37:51)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K74"/>
+  <dimension ref="A1:K77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1584,11 +1584,7 @@
           <t xml:space="preserve">26/May - Requisición Aun no se tiene autorización 21485 - HERRAMENTAL DOBLEZ </t>
         </is>
       </c>
-      <c r="K24" s="3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -1682,11 +1678,7 @@
           <t>28/May - Se a reenviado las Requisiciones al Ing. Alfredo para autorización 21348-21092</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -2103,11 +2095,7 @@
           <t>28/May - Solicitud eviada al Ing. Alfredo de PC para Ing. Rodolfo.</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -3912,6 +3900,142 @@
       </c>
       <c r="J74" t="inlineStr"/>
       <c r="K74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Programa de Actividades</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>09-Jun-26</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Cruz Carreon</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>🔍 Calidad</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Fabricar Mesa para Nonio de Calidad revisión Dimensional.</t>
+        </is>
+      </c>
+      <c r="H75" t="n">
+        <v>0</v>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>12-Jun-26</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Mejoras</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>09-Jun-26</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Jesus Morales</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>👥 Recursos Humanos</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Mejorar Reporte y agregar Historico de Semanas en una nueva Base de Datos dentro de la Aplicación.</t>
+        </is>
+      </c>
+      <c r="H76" t="n">
+        <v>0</v>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>12-Jun-26</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Programa de Actividades</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>09-Jun-26</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Jesus Morales</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>✂️ Corte</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pre-programa para aplicación de WiP Area de Corte Laser.
+</t>
+        </is>
+      </c>
+      <c r="H77" t="n">
+        <v>0</v>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>12-Jun-26</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-06-17 23:13:40)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -47,12 +47,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8D7DA"/>
+        <fgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF3CD"/>
+        <fgColor rgb="00F8D7DA"/>
       </patternFill>
     </fill>
   </fills>
@@ -71,8 +71,8 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K77"/>
+  <dimension ref="A1:K81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1060,53 +1060,49 @@
       <c r="K13" s="1" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>Mejoras</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F14" s="1" t="inlineStr">
         <is>
           <t>📐 Doblez</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G14" s="1" t="inlineStr">
         <is>
           <t>Cotizar Refacciones de maquinas Dobladoras</t>
         </is>
       </c>
-      <c r="H14" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="H14" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I14" s="1" t="inlineStr">
         <is>
           <t>5-Jun-26</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>12/May - Se mando Correo a Flex con Imágenes</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr"/>
+      <c r="J14" s="1" t="inlineStr"/>
+      <c r="K14" s="1" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -1399,53 +1395,53 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n">
+      <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Auto Asignado</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>11-May-26</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>👑 Direccion</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>Autorización compra de aspiradora para limpieza de Lijadora</t>
         </is>
       </c>
-      <c r="H21" s="3" t="n">
+      <c r="H21" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="I21" s="3" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>27-Jun-26</t>
         </is>
       </c>
-      <c r="J21" s="3" t="inlineStr">
+      <c r="J21" s="2" t="inlineStr">
         <is>
           <t>26/May - Requisición en SAI  21396 - REQ. HTA. PARTE 2JM</t>
         </is>
       </c>
-      <c r="K21" s="3" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -1538,53 +1534,53 @@
       <c r="K23" s="1" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="n">
+      <c r="A24" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>12-May-26</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>👑 Direccion</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>Autorización de Matriz Dobladora 85x85x3200</t>
         </is>
       </c>
-      <c r="H24" s="3" t="n">
+      <c r="H24" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="I24" s="3" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>27-Jun-26</t>
         </is>
       </c>
-      <c r="J24" s="3" t="inlineStr">
+      <c r="J24" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">26/May - Requisición Aun no se tiene autorización 21485 - HERRAMENTAL DOBLEZ </t>
         </is>
       </c>
-      <c r="K24" s="3" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -1726,49 +1722,49 @@
       <c r="K27" s="1" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n">
+      <c r="A28" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>12-May-26</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E28" s="3" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F28" s="3" t="inlineStr">
         <is>
           <t>📐 Doblez</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>Diseño de Carro de Herramental Doblez</t>
         </is>
       </c>
-      <c r="H28" s="2" t="n">
+      <c r="H28" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="I28" s="2" t="inlineStr">
+      <c r="I28" s="3" t="inlineStr">
         <is>
           <t>5-Jun-26</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr"/>
+      <c r="J28" s="3" t="inlineStr"/>
+      <c r="K28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -2000,53 +1996,53 @@
       <c r="K33" s="1" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" t="n">
+      <c r="A34" s="1" t="n">
         <v>33</v>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="1" t="inlineStr">
         <is>
           <t>25-May-26</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
+      <c r="D34" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E34" s="1" t="inlineStr">
         <is>
           <t>Luis Quintana</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F34" s="1" t="inlineStr">
         <is>
           <t>📦 Almacen</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G34" s="1" t="inlineStr">
         <is>
           <t>Requisición de Quimicos para lineas de Pintura</t>
         </is>
       </c>
-      <c r="H34" t="n">
-        <v>50</v>
-      </c>
-      <c r="I34" t="inlineStr">
+      <c r="H34" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I34" s="1" t="inlineStr">
         <is>
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="J34" s="1" t="inlineStr">
         <is>
           <t>03/Jun - Requisición Seguimiento</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr"/>
+      <c r="K34" s="1" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2098,53 +2094,57 @@
       <c r="K35" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" t="n">
+      <c r="A36" s="1" t="n">
         <v>35</v>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="1" t="inlineStr">
         <is>
           <t>Dirección</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="1" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
+      <c r="D36" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E36" s="1" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F36" s="1" t="inlineStr">
         <is>
           <t>👑 Direccion</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G36" s="1" t="inlineStr">
         <is>
           <t>Capacitar en sistema SAI para hacer Requisiciones en Sistema.</t>
         </is>
       </c>
-      <c r="H36" t="n">
-        <v>0</v>
-      </c>
-      <c r="I36" t="inlineStr">
+      <c r="H36" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I36" s="1" t="inlineStr">
         <is>
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="J36" s="1" t="inlineStr">
         <is>
           <t>28/May - Se programa para Viernes 29 a las 10:00 a,m,</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr"/>
+      <c r="K36" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -2576,143 +2576,143 @@
       <c r="K45" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n">
+      <c r="A46" s="1" t="n">
         <v>45</v>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B46" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="C46" s="1" t="inlineStr">
         <is>
           <t>28-May-26</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="D46" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E46" s="1" t="inlineStr">
         <is>
           <t>Luis Quintana</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F46" s="1" t="inlineStr">
         <is>
           <t>🚚 Embarquez</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G46" s="1" t="inlineStr">
         <is>
           <t>26/May  - Comenzar el proceso de empaquetado del Material en DIAGONAL 1600 piezas</t>
         </is>
       </c>
-      <c r="H46" s="2" t="n">
+      <c r="H46" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I46" s="1" t="inlineStr">
+        <is>
+          <t>05-Jun-26</t>
+        </is>
+      </c>
+      <c r="J46" s="1" t="inlineStr">
+        <is>
+          <t>03/Jun - Avance 70%</t>
+        </is>
+      </c>
+      <c r="K46" s="1" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="1" t="inlineStr">
+        <is>
+          <t>Dirección</t>
+        </is>
+      </c>
+      <c r="C47" s="1" t="inlineStr">
+        <is>
+          <t>28-May-26</t>
+        </is>
+      </c>
+      <c r="D47" s="1" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E47" s="1" t="inlineStr">
+        <is>
+          <t>Luis Quintana</t>
+        </is>
+      </c>
+      <c r="F47" s="1" t="inlineStr">
+        <is>
+          <t>📦 Almacen</t>
+        </is>
+      </c>
+      <c r="G47" s="1" t="inlineStr">
+        <is>
+          <t>Reubicar los racks a la pared bajo el Extractor.</t>
+        </is>
+      </c>
+      <c r="H47" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I47" s="1" t="inlineStr">
+        <is>
+          <t>05-Jun-26</t>
+        </is>
+      </c>
+      <c r="J47" s="1" t="inlineStr"/>
+      <c r="K47" s="1" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Programa de Actividades</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>28-May-26</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Rodolfo Ferndez M</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>⚙️ Ingenieria</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>Elaborar el primer procedimiento de Ingenieria para primera pieza segén el proceso actual</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="n">
         <v>70</v>
       </c>
-      <c r="I46" s="2" t="inlineStr">
+      <c r="I48" s="3" t="inlineStr">
         <is>
           <t>05-Jun-26</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>03/Jun - Avance 70%</t>
-        </is>
-      </c>
-      <c r="K46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="n">
-        <v>46</v>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>Dirección</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>28-May-26</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>Luis Quintana</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>📦 Almacen</t>
-        </is>
-      </c>
-      <c r="G47" s="2" t="inlineStr">
-        <is>
-          <t>Reubicar los racks a la pared bajo el Extractor.</t>
-        </is>
-      </c>
-      <c r="H47" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I47" s="2" t="inlineStr">
-        <is>
-          <t>05-Jun-26</t>
-        </is>
-      </c>
-      <c r="J47" s="2" t="inlineStr"/>
-      <c r="K47" s="2" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="n">
-        <v>47</v>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Programa de Actividades</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>28-May-26</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>Rodolfo Ferndez M</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>⚙️ Ingenieria</t>
-        </is>
-      </c>
-      <c r="G48" s="2" t="inlineStr">
-        <is>
-          <t>Elaborar el primer procedimiento de Ingenieria para primera pieza segén el proceso actual</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t>05-Jun-26</t>
-        </is>
-      </c>
-      <c r="J48" s="2" t="inlineStr"/>
-      <c r="K48" s="2" t="inlineStr"/>
+      <c r="J48" s="3" t="inlineStr"/>
+      <c r="K48" s="3" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
@@ -2948,49 +2948,49 @@
       <c r="K53" s="1" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n">
+      <c r="A54" s="3" t="n">
         <v>53</v>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B54" s="3" t="inlineStr">
         <is>
           <t>Mejoras</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
+      <c r="C54" s="3" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F54" s="3" t="inlineStr">
         <is>
           <t>📐 Doblez</t>
         </is>
       </c>
-      <c r="G54" s="2" t="inlineStr">
+      <c r="G54" s="3" t="inlineStr">
         <is>
           <t>Hacer requisición de Grasa para maquinas Dobladoras (Cremayeras)</t>
         </is>
       </c>
-      <c r="H54" s="2" t="n">
+      <c r="H54" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I54" s="2" t="inlineStr">
+      <c r="I54" s="3" t="inlineStr">
         <is>
           <t>05-Jun-26</t>
         </is>
       </c>
-      <c r="J54" s="2" t="inlineStr"/>
-      <c r="K54" s="2" t="inlineStr"/>
+      <c r="J54" s="3" t="inlineStr"/>
+      <c r="K54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
@@ -3128,139 +3128,139 @@
       <c r="K57" s="1" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" t="n">
+      <c r="A58" s="3" t="n">
         <v>57</v>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B58" s="3" t="inlineStr">
         <is>
           <t>Mejoras</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C58" s="3" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D58" s="3" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="E58" s="3" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="F58" s="3" t="inlineStr">
         <is>
           <t>⚙️ Ingenieria</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr">
+      <c r="G58" s="3" t="inlineStr">
         <is>
           <t>Instalar Interruptor de Extractor</t>
         </is>
       </c>
-      <c r="H58" t="n">
+      <c r="H58" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I58" t="inlineStr">
+      <c r="I58" s="3" t="inlineStr">
         <is>
           <t>12-Jun-26</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
+      <c r="J58" s="3" t="inlineStr"/>
+      <c r="K58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n">
+      <c r="A59" s="3" t="n">
         <v>58</v>
       </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="D59" s="3" t="inlineStr">
         <is>
           <t>Urgente</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="E59" s="3" t="inlineStr">
         <is>
           <t>Luis Quintana</t>
         </is>
       </c>
-      <c r="F59" s="2" t="inlineStr">
+      <c r="F59" s="3" t="inlineStr">
         <is>
           <t>🚚 Embarquez</t>
         </is>
       </c>
-      <c r="G59" s="2" t="inlineStr">
+      <c r="G59" s="3" t="inlineStr">
         <is>
           <t>Elaborar Lista de Reposiciones para Proyecto Reno 6 Parcialidad 2.- Despues de Inventario</t>
         </is>
       </c>
-      <c r="H59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I59" s="2" t="inlineStr">
+      <c r="H59" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
         <is>
           <t>04-Jun-26</t>
         </is>
       </c>
-      <c r="J59" s="2" t="inlineStr"/>
-      <c r="K59" s="2" t="inlineStr"/>
+      <c r="J59" s="3" t="inlineStr"/>
+      <c r="K59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n">
+      <c r="A60" s="3" t="n">
         <v>59</v>
       </c>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="B60" s="3" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
+      <c r="C60" s="3" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="D60" s="3" t="inlineStr">
         <is>
           <t>Urgente</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="E60" s="3" t="inlineStr">
         <is>
           <t>Luis Quintana</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr">
+      <c r="F60" s="3" t="inlineStr">
         <is>
           <t>🚚 Embarquez</t>
         </is>
       </c>
-      <c r="G60" s="2" t="inlineStr">
+      <c r="G60" s="3" t="inlineStr">
         <is>
           <t>Lista de Reposiciones Reno 6 Parcialodad 2</t>
         </is>
       </c>
-      <c r="H60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I60" s="2" t="inlineStr">
+      <c r="H60" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="I60" s="3" t="inlineStr">
         <is>
           <t>04-Jun-26</t>
         </is>
       </c>
-      <c r="J60" s="2" t="inlineStr"/>
-      <c r="K60" s="2" t="inlineStr"/>
+      <c r="J60" s="3" t="inlineStr"/>
+      <c r="K60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
@@ -3402,274 +3402,274 @@
       <c r="K63" s="1" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n">
+      <c r="A64" s="3" t="n">
         <v>63</v>
       </c>
-      <c r="B64" s="2" t="inlineStr">
+      <c r="B64" s="3" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
+      <c r="C64" s="3" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D64" s="2" t="inlineStr">
+      <c r="D64" s="3" t="inlineStr">
         <is>
           <t>Urgente</t>
         </is>
       </c>
-      <c r="E64" s="2" t="inlineStr">
+      <c r="E64" s="3" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F64" s="2" t="inlineStr">
+      <c r="F64" s="3" t="inlineStr">
         <is>
           <t>✂️ Corte</t>
         </is>
       </c>
-      <c r="G64" s="2" t="inlineStr">
+      <c r="G64" s="3" t="inlineStr">
         <is>
           <t>Definir y Generar el WIP #1  Pos-laser</t>
         </is>
       </c>
-      <c r="H64" s="2" t="n">
+      <c r="H64" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I64" s="2" t="inlineStr">
+      <c r="I64" s="3" t="inlineStr">
         <is>
           <t>08-Jun-26</t>
         </is>
       </c>
-      <c r="J64" s="2" t="inlineStr"/>
-      <c r="K64" s="2" t="inlineStr"/>
+      <c r="J64" s="3" t="inlineStr"/>
+      <c r="K64" s="3" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" t="n">
+      <c r="A65" s="3" t="n">
         <v>64</v>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B65" s="3" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C65" s="3" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr">
+      <c r="D65" s="3" t="inlineStr">
         <is>
           <t>Urgente</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
+      <c r="E65" s="3" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="F65" s="3" t="inlineStr">
         <is>
           <t>✂️ Corte</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr">
+      <c r="G65" s="3" t="inlineStr">
         <is>
           <t>Impacto de Wip en Procedimiento</t>
         </is>
       </c>
-      <c r="H65" t="n">
+      <c r="H65" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I65" t="inlineStr">
+      <c r="I65" s="3" t="inlineStr">
         <is>
           <t>12-Jun-26</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
+      <c r="J65" s="3" t="inlineStr"/>
+      <c r="K65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" t="n">
+      <c r="A66" s="3" t="n">
         <v>65</v>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B66" s="3" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C66" s="3" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="D66" s="3" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
+      <c r="E66" s="3" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr">
+      <c r="F66" s="3" t="inlineStr">
         <is>
           <t>✂️ Corte</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr">
+      <c r="G66" s="3" t="inlineStr">
         <is>
           <t>Archivos de Programa de Producción por Estación</t>
         </is>
       </c>
-      <c r="H66" t="n">
+      <c r="H66" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I66" t="inlineStr">
+      <c r="I66" s="3" t="inlineStr">
         <is>
           <t>12-Jun-26</t>
         </is>
       </c>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
+      <c r="J66" s="3" t="inlineStr"/>
+      <c r="K66" s="3" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n">
+      <c r="A67" s="3" t="n">
         <v>66</v>
       </c>
-      <c r="B67" s="2" t="inlineStr">
+      <c r="B67" s="3" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr">
+      <c r="C67" s="3" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
         <is>
           <t>Rodolfo Ferndez M</t>
         </is>
       </c>
-      <c r="F67" s="2" t="inlineStr">
+      <c r="F67" s="3" t="inlineStr">
         <is>
           <t>⚙️ Ingenieria</t>
         </is>
       </c>
-      <c r="G67" s="2" t="inlineStr">
+      <c r="G67" s="3" t="inlineStr">
         <is>
           <t>Revisión Con Cruz y Bryan del Procedimiento de Ingenieria</t>
         </is>
       </c>
-      <c r="H67" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I67" s="2" t="inlineStr">
+      <c r="H67" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="I67" s="3" t="inlineStr">
         <is>
           <t>05-Jun-26</t>
         </is>
       </c>
-      <c r="J67" s="2" t="inlineStr"/>
-      <c r="K67" s="2" t="inlineStr"/>
+      <c r="J67" s="3" t="inlineStr"/>
+      <c r="K67" s="3" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" t="n">
+      <c r="A68" s="3" t="n">
         <v>67</v>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B68" s="3" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C68" s="3" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
         <is>
           <t>Rodolfo Ferndez M</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr">
+      <c r="F68" s="3" t="inlineStr">
         <is>
           <t>⚙️ Ingenieria</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr">
+      <c r="G68" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Revisión Con Area de Calidad del Procedimiento </t>
         </is>
       </c>
-      <c r="H68" t="n">
-        <v>0</v>
-      </c>
-      <c r="I68" t="inlineStr">
+      <c r="H68" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="I68" s="3" t="inlineStr">
         <is>
           <t>12-Jun-26</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
+      <c r="J68" s="3" t="inlineStr"/>
+      <c r="K68" s="3" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" t="n">
+      <c r="A69" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="B69" t="inlineStr">
+      <c r="B69" s="2" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
         <is>
           <t>Rodolfo Ferndez M</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr">
+      <c r="F69" s="2" t="inlineStr">
         <is>
           <t>⚙️ Ingenieria</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr">
+      <c r="G69" s="2" t="inlineStr">
         <is>
           <t>Actualización de Planos Armando WOO Aprox. 70 Planos.</t>
         </is>
       </c>
-      <c r="H69" t="n">
-        <v>0</v>
-      </c>
-      <c r="I69" t="inlineStr">
+      <c r="H69" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
         <is>
           <t>19-Jun-26</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
+      <c r="J69" s="2" t="inlineStr"/>
+      <c r="K69" s="2" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
@@ -3857,185 +3857,377 @@
       <c r="K73" s="1" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" t="n">
+      <c r="A74" s="1" t="n">
         <v>73</v>
       </c>
-      <c r="B74" t="inlineStr">
+      <c r="B74" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
+      <c r="C74" s="1" t="inlineStr">
         <is>
           <t>08-Jun-26</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
+      <c r="D74" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E74" s="1" t="inlineStr">
         <is>
           <t>Luis Quintana</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr">
+      <c r="F74" s="1" t="inlineStr">
         <is>
           <t>🚚 Embarquez</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr">
+      <c r="G74" s="1" t="inlineStr">
         <is>
           <t>Generar Correo electronico de la Primera Remisión Generada en Programa de METALES.</t>
         </is>
       </c>
-      <c r="H74" t="n">
-        <v>0</v>
-      </c>
-      <c r="I74" t="inlineStr">
+      <c r="H74" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I74" s="1" t="inlineStr">
         <is>
           <t>12-Jun-26</t>
         </is>
       </c>
-      <c r="J74" t="inlineStr"/>
-      <c r="K74" t="inlineStr"/>
+      <c r="J74" s="1" t="inlineStr"/>
+      <c r="K74" s="1" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" t="n">
+      <c r="A75" s="1" t="n">
         <v>74</v>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B75" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C75" s="1" t="inlineStr">
         <is>
           <t>09-Jun-26</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
+      <c r="D75" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E75" s="1" t="inlineStr">
         <is>
           <t>Cruz Carreon</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr">
+      <c r="F75" s="1" t="inlineStr">
         <is>
           <t>🔍 Calidad</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr">
+      <c r="G75" s="1" t="inlineStr">
         <is>
           <t>Fabricar Mesa para Nonio de Calidad revisión Dimensional.</t>
         </is>
       </c>
-      <c r="H75" t="n">
-        <v>0</v>
-      </c>
-      <c r="I75" t="inlineStr">
+      <c r="H75" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I75" s="1" t="inlineStr">
         <is>
           <t>12-Jun-26</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr"/>
+      <c r="J75" s="1" t="inlineStr"/>
+      <c r="K75" s="1" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" t="n">
+      <c r="A76" s="1" t="n">
         <v>75</v>
       </c>
-      <c r="B76" t="inlineStr">
+      <c r="B76" s="1" t="inlineStr">
         <is>
           <t>Mejoras</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C76" s="1" t="inlineStr">
         <is>
           <t>09-Jun-26</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr">
+      <c r="D76" s="1" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
+      <c r="E76" s="1" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
+      <c r="F76" s="1" t="inlineStr">
         <is>
           <t>👥 Recursos Humanos</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr">
+      <c r="G76" s="1" t="inlineStr">
         <is>
           <t>Mejorar Reporte y agregar Historico de Semanas en una nueva Base de Datos dentro de la Aplicación.</t>
         </is>
       </c>
-      <c r="H76" t="n">
-        <v>0</v>
-      </c>
-      <c r="I76" t="inlineStr">
+      <c r="H76" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I76" s="1" t="inlineStr">
         <is>
           <t>12-Jun-26</t>
         </is>
       </c>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr"/>
+      <c r="J76" s="1" t="inlineStr"/>
+      <c r="K76" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="77">
-      <c r="A77" t="n">
+      <c r="A77" s="3" t="n">
         <v>76</v>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B77" s="3" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C77" s="3" t="inlineStr">
         <is>
           <t>09-Jun-26</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr">
+      <c r="F77" s="3" t="inlineStr">
         <is>
           <t>✂️ Corte</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr">
+      <c r="G77" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Pre-programa para aplicación de WiP Area de Corte Laser.
 </t>
         </is>
       </c>
-      <c r="H77" t="n">
+      <c r="H77" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="I77" s="3" t="inlineStr">
+        <is>
+          <t>12-Jun-26</t>
+        </is>
+      </c>
+      <c r="J77" s="3" t="inlineStr"/>
+      <c r="K77" s="3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="1" t="inlineStr">
+        <is>
+          <t>Acuerdos</t>
+        </is>
+      </c>
+      <c r="C78" s="1" t="inlineStr">
+        <is>
+          <t>15-Jun-26</t>
+        </is>
+      </c>
+      <c r="D78" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E78" s="1" t="inlineStr">
+        <is>
+          <t>Jesus Morales</t>
+        </is>
+      </c>
+      <c r="F78" s="1" t="inlineStr">
+        <is>
+          <t>🔍 Calidad</t>
+        </is>
+      </c>
+      <c r="G78" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Generar Aplicación para Incomming de Materia Prima:  </t>
+        </is>
+      </c>
+      <c r="H78" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I78" s="1" t="inlineStr">
+        <is>
+          <t>19-Jun-26</t>
+        </is>
+      </c>
+      <c r="J78" s="1" t="inlineStr"/>
+      <c r="K78" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Dirección</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>16-Jun-26</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Bryan Flores</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>✂️ Corte</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Definición de ACRONIMO y DISEÑO de orden de trabajo para Corte LASER. </t>
+        </is>
+      </c>
+      <c r="H79" t="n">
         <v>0</v>
       </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>12-Jun-26</t>
-        </is>
-      </c>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>19-Jun-26</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Procesos</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>16-Jun-26</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Rodolfo Ferndez M</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>⚙️ Ingenieria</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Presentar al equipo de calidad, corte y doblez el procedimiento de aprobación de primera pieza</t>
+        </is>
+      </c>
+      <c r="H80" t="n">
+        <v>0</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>18-Jun-26</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Procesos</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>16-Jun-26</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Rodolfo Ferndez M</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>⚙️ Ingenieria</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Presentar al equipo de calidad, corte y doblez el procedimiento de aprobación de primera pieza</t>
+        </is>
+      </c>
+      <c r="H81" t="n">
+        <v>0</v>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>18-Jun-26</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-06-17 23:14:47)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K81"/>
+  <dimension ref="A1:K80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4184,51 +4184,6 @@
       <c r="J80" t="inlineStr"/>
       <c r="K80" t="inlineStr"/>
     </row>
-    <row r="81">
-      <c r="A81" t="n">
-        <v>80</v>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>Procesos</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>16-Jun-26</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>Rodolfo Ferndez M</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>⚙️ Ingenieria</t>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>Presentar al equipo de calidad, corte y doblez el procedimiento de aprobación de primera pieza</t>
-        </is>
-      </c>
-      <c r="H81" t="n">
-        <v>0</v>
-      </c>
-      <c r="I81" t="inlineStr">
-        <is>
-          <t>18-Jun-26</t>
-        </is>
-      </c>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-06-18 18:08:02)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -2140,11 +2140,7 @@
           <t>28/May - Se programa para Viernes 29 a las 10:00 a,m,</t>
         </is>
       </c>
-      <c r="K36" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K36" s="1" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -3989,61 +3985,53 @@
         </is>
       </c>
       <c r="J76" s="1" t="inlineStr"/>
-      <c r="K76" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K76" s="1" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="3" t="n">
+      <c r="A77" s="2" t="n">
         <v>76</v>
       </c>
-      <c r="B77" s="3" t="inlineStr">
+      <c r="B77" s="2" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C77" s="3" t="inlineStr">
+      <c r="C77" s="2" t="inlineStr">
         <is>
           <t>09-Jun-26</t>
         </is>
       </c>
-      <c r="D77" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E77" s="3" t="inlineStr">
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
         <is>
           <t>Jesus Morales</t>
         </is>
       </c>
-      <c r="F77" s="3" t="inlineStr">
+      <c r="F77" s="2" t="inlineStr">
         <is>
           <t>✂️ Corte</t>
         </is>
       </c>
-      <c r="G77" s="3" t="inlineStr">
+      <c r="G77" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Pre-programa para aplicación de WiP Area de Corte Laser.
 </t>
         </is>
       </c>
-      <c r="H77" s="3" t="n">
+      <c r="H77" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="I77" s="3" t="inlineStr">
-        <is>
-          <t>12-Jun-26</t>
-        </is>
-      </c>
-      <c r="J77" s="3" t="inlineStr"/>
-      <c r="K77" s="3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>30-Jun-26</t>
+        </is>
+      </c>
+      <c r="J77" s="2" t="inlineStr"/>
+      <c r="K77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
@@ -4088,11 +4076,7 @@
         </is>
       </c>
       <c r="J78" s="1" t="inlineStr"/>
-      <c r="K78" s="1" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="K78" s="1" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -4140,49 +4124,49 @@
       <c r="K79" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" t="n">
+      <c r="A80" s="3" t="n">
         <v>79</v>
       </c>
-      <c r="B80" t="inlineStr">
+      <c r="B80" s="3" t="inlineStr">
         <is>
           <t>Procesos</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr">
+      <c r="C80" s="3" t="inlineStr">
         <is>
           <t>16-Jun-26</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr">
+      <c r="D80" s="3" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr">
+      <c r="E80" s="3" t="inlineStr">
         <is>
           <t>Rodolfo Ferndez M</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr">
+      <c r="F80" s="3" t="inlineStr">
         <is>
           <t>⚙️ Ingenieria</t>
         </is>
       </c>
-      <c r="G80" t="inlineStr">
+      <c r="G80" s="3" t="inlineStr">
         <is>
           <t>Presentar al equipo de calidad, corte y doblez el procedimiento de aprobación de primera pieza</t>
         </is>
       </c>
-      <c r="H80" t="n">
+      <c r="H80" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I80" t="inlineStr">
+      <c r="I80" s="3" t="inlineStr">
         <is>
           <t>18-Jun-26</t>
         </is>
       </c>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
+      <c r="J80" s="3" t="inlineStr"/>
+      <c r="K80" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-06-18 18:09:55)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -2666,49 +2666,53 @@
       <c r="K47" s="1" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="3" t="n">
+      <c r="A48" s="1" t="n">
         <v>47</v>
       </c>
-      <c r="B48" s="3" t="inlineStr">
+      <c r="B48" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C48" s="3" t="inlineStr">
+      <c r="C48" s="1" t="inlineStr">
         <is>
           <t>28-May-26</t>
         </is>
       </c>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E48" s="3" t="inlineStr">
+      <c r="D48" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E48" s="1" t="inlineStr">
         <is>
           <t>Rodolfo Ferndez M</t>
         </is>
       </c>
-      <c r="F48" s="3" t="inlineStr">
+      <c r="F48" s="1" t="inlineStr">
         <is>
           <t>⚙️ Ingenieria</t>
         </is>
       </c>
-      <c r="G48" s="3" t="inlineStr">
+      <c r="G48" s="1" t="inlineStr">
         <is>
           <t>Elaborar el primer procedimiento de Ingenieria para primera pieza segén el proceso actual</t>
         </is>
       </c>
-      <c r="H48" s="3" t="n">
-        <v>70</v>
-      </c>
-      <c r="I48" s="3" t="inlineStr">
+      <c r="H48" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I48" s="1" t="inlineStr">
         <is>
           <t>05-Jun-26</t>
         </is>
       </c>
-      <c r="J48" s="3" t="inlineStr"/>
-      <c r="K48" s="3" t="inlineStr"/>
+      <c r="J48" s="1" t="inlineStr"/>
+      <c r="K48" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
@@ -3533,49 +3537,53 @@
       <c r="K66" s="3" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="3" t="n">
+      <c r="A67" s="1" t="n">
         <v>66</v>
       </c>
-      <c r="B67" s="3" t="inlineStr">
+      <c r="B67" s="1" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C67" s="3" t="inlineStr">
+      <c r="C67" s="1" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D67" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E67" s="3" t="inlineStr">
+      <c r="D67" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E67" s="1" t="inlineStr">
         <is>
           <t>Rodolfo Ferndez M</t>
         </is>
       </c>
-      <c r="F67" s="3" t="inlineStr">
+      <c r="F67" s="1" t="inlineStr">
         <is>
           <t>⚙️ Ingenieria</t>
         </is>
       </c>
-      <c r="G67" s="3" t="inlineStr">
+      <c r="G67" s="1" t="inlineStr">
         <is>
           <t>Revisión Con Cruz y Bryan del Procedimiento de Ingenieria</t>
         </is>
       </c>
-      <c r="H67" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="I67" s="3" t="inlineStr">
+      <c r="H67" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I67" s="1" t="inlineStr">
         <is>
           <t>05-Jun-26</t>
         </is>
       </c>
-      <c r="J67" s="3" t="inlineStr"/>
-      <c r="K67" s="3" t="inlineStr"/>
+      <c r="J67" s="1" t="inlineStr"/>
+      <c r="K67" s="1" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="n">
@@ -3657,7 +3665,7 @@
         </is>
       </c>
       <c r="H69" s="2" t="n">
-        <v>60</v>
+        <v>85</v>
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
@@ -3665,7 +3673,11 @@
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr"/>
-      <c r="K69" s="2" t="inlineStr"/>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-06-18 18:11:46)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -3402,139 +3402,139 @@
       <c r="K63" s="1" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="3" t="n">
+      <c r="A64" t="n">
         <v>63</v>
       </c>
-      <c r="B64" s="3" t="inlineStr">
+      <c r="B64" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C64" s="3" t="inlineStr">
+      <c r="C64" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D64" s="3" t="inlineStr">
+      <c r="D64" t="inlineStr">
         <is>
           <t>Urgente</t>
         </is>
       </c>
-      <c r="E64" s="3" t="inlineStr">
+      <c r="E64" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F64" s="3" t="inlineStr">
+      <c r="F64" t="inlineStr">
         <is>
           <t>✂️ Corte</t>
         </is>
       </c>
-      <c r="G64" s="3" t="inlineStr">
+      <c r="G64" t="inlineStr">
         <is>
           <t>Definir y Generar el WIP #1  Pos-laser</t>
         </is>
       </c>
-      <c r="H64" s="3" t="n">
+      <c r="H64" t="n">
         <v>0</v>
       </c>
-      <c r="I64" s="3" t="inlineStr">
-        <is>
-          <t>08-Jun-26</t>
-        </is>
-      </c>
-      <c r="J64" s="3" t="inlineStr"/>
-      <c r="K64" s="3" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>30-Jun-26</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="3" t="n">
+      <c r="A65" t="n">
         <v>64</v>
       </c>
-      <c r="B65" s="3" t="inlineStr">
+      <c r="B65" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C65" s="3" t="inlineStr">
+      <c r="C65" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D65" s="3" t="inlineStr">
+      <c r="D65" t="inlineStr">
         <is>
           <t>Urgente</t>
         </is>
       </c>
-      <c r="E65" s="3" t="inlineStr">
+      <c r="E65" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F65" s="3" t="inlineStr">
+      <c r="F65" t="inlineStr">
         <is>
           <t>✂️ Corte</t>
         </is>
       </c>
-      <c r="G65" s="3" t="inlineStr">
+      <c r="G65" t="inlineStr">
         <is>
           <t>Impacto de Wip en Procedimiento</t>
         </is>
       </c>
-      <c r="H65" s="3" t="n">
+      <c r="H65" t="n">
         <v>0</v>
       </c>
-      <c r="I65" s="3" t="inlineStr">
-        <is>
-          <t>12-Jun-26</t>
-        </is>
-      </c>
-      <c r="J65" s="3" t="inlineStr"/>
-      <c r="K65" s="3" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>30-Jun-26</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="3" t="n">
+      <c r="A66" t="n">
         <v>65</v>
       </c>
-      <c r="B66" s="3" t="inlineStr">
+      <c r="B66" t="inlineStr">
         <is>
           <t>Problema de Calidad</t>
         </is>
       </c>
-      <c r="C66" s="3" t="inlineStr">
+      <c r="C66" t="inlineStr">
         <is>
           <t>03-Jun-26</t>
         </is>
       </c>
-      <c r="D66" s="3" t="inlineStr">
+      <c r="D66" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E66" s="3" t="inlineStr">
+      <c r="E66" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F66" s="3" t="inlineStr">
+      <c r="F66" t="inlineStr">
         <is>
           <t>✂️ Corte</t>
         </is>
       </c>
-      <c r="G66" s="3" t="inlineStr">
+      <c r="G66" t="inlineStr">
         <is>
           <t>Archivos de Programa de Producción por Estación</t>
         </is>
       </c>
-      <c r="H66" s="3" t="n">
+      <c r="H66" t="n">
         <v>0</v>
       </c>
-      <c r="I66" s="3" t="inlineStr">
-        <is>
-          <t>12-Jun-26</t>
-        </is>
-      </c>
-      <c r="J66" s="3" t="inlineStr"/>
-      <c r="K66" s="3" t="inlineStr"/>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>30-Jun-26</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">

</xml_diff>

<commit_message>
Seccion Cargar Actividades: lista inferior ordenada con las 5 ultimas en amarillo, y resumen de registro validado con fecha, responsable, nombre y tiempo de ejecucion
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="177">
   <si>
     <t>No</t>
   </si>
@@ -538,6 +538,9 @@
   </si>
   <si>
     <t>evidencias/MCE-019_evidencia.jpg</t>
+  </si>
+  <si>
+    <t>nan</t>
   </si>
   <si>
     <t>evidencias/MCE-041_evidencia_20260608_225041.jpg</t>
@@ -1516,6 +1519,9 @@
       <c r="J21" t="s">
         <v>157</v>
       </c>
+      <c r="K21" t="s">
+        <v>174</v>
+      </c>
     </row>
     <row r="22" spans="1:11">
       <c r="A22">
@@ -2153,7 +2159,7 @@
         <v>166</v>
       </c>
       <c r="K42" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="43" spans="1:11">
@@ -2986,7 +2992,7 @@
         <v>29</v>
       </c>
       <c r="K70" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="71" spans="1:11">

</xml_diff>

<commit_message>
Mover resumen de validacion de registro debajo del boton de Registrar Actividad
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="596" uniqueCount="178">
   <si>
     <t>No</t>
   </si>
@@ -110,6 +110,9 @@
   </si>
   <si>
     <t>16-Jun-26</t>
+  </si>
+  <si>
+    <t>22-Jun-26</t>
   </si>
   <si>
     <t>Media</t>
@@ -405,6 +408,9 @@
     <t>Presentar al equipo de calidad, corte y doblez el procedimiento de aprobación de primera pieza</t>
   </si>
   <si>
+    <t>Actualización de APP, Mejoras con Imagen Corporativa.</t>
+  </si>
+  <si>
     <t>15-May-26</t>
   </si>
   <si>
@@ -538,9 +544,6 @@
   </si>
   <si>
     <t>evidencias/MCE-019_evidencia.jpg</t>
-  </si>
-  <si>
-    <t>nan</t>
   </si>
   <si>
     <t>evidencias/MCE-041_evidencia_20260608_225041.jpg</t>
@@ -878,7 +881,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K80"/>
+  <dimension ref="A1:K81"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
@@ -927,16 +930,16 @@
         <v>19</v>
       </c>
       <c r="D2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H2">
         <v>100</v>
@@ -945,7 +948,7 @@
         <v>19</v>
       </c>
       <c r="J2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -959,22 +962,22 @@
         <v>19</v>
       </c>
       <c r="D3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H3">
         <v>100</v>
       </c>
       <c r="I3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -988,22 +991,22 @@
         <v>19</v>
       </c>
       <c r="D4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H4">
         <v>100</v>
       </c>
       <c r="I4" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -1017,22 +1020,22 @@
         <v>19</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H5">
         <v>100</v>
       </c>
       <c r="I5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -1046,22 +1049,22 @@
         <v>19</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H6">
         <v>100</v>
       </c>
       <c r="I6" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -1075,22 +1078,22 @@
         <v>19</v>
       </c>
       <c r="D7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H7">
         <v>100</v>
       </c>
       <c r="I7" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -1104,22 +1107,22 @@
         <v>19</v>
       </c>
       <c r="D8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H8">
         <v>100</v>
       </c>
       <c r="I8" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -1133,25 +1136,25 @@
         <v>19</v>
       </c>
       <c r="D9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H9">
         <v>100</v>
       </c>
       <c r="I9" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="J9" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -1165,22 +1168,22 @@
         <v>19</v>
       </c>
       <c r="D10" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H10">
         <v>100</v>
       </c>
       <c r="I10" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -1194,22 +1197,22 @@
         <v>19</v>
       </c>
       <c r="D11" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F11" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G11" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H11">
         <v>100</v>
       </c>
       <c r="I11" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -1223,22 +1226,22 @@
         <v>19</v>
       </c>
       <c r="D12" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H12">
         <v>100</v>
       </c>
       <c r="I12" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -1252,22 +1255,22 @@
         <v>19</v>
       </c>
       <c r="D13" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F13" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H13">
         <v>100</v>
       </c>
       <c r="I13" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -1281,22 +1284,22 @@
         <v>19</v>
       </c>
       <c r="D14" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E14" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F14" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H14">
         <v>100</v>
       </c>
       <c r="I14" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -1310,25 +1313,25 @@
         <v>19</v>
       </c>
       <c r="D15" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E15" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F15" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G15" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H15">
         <v>100</v>
       </c>
       <c r="I15" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="J15" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -1342,25 +1345,25 @@
         <v>19</v>
       </c>
       <c r="D16" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E16" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G16" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H16">
         <v>100</v>
       </c>
       <c r="I16" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="J16" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -1374,25 +1377,25 @@
         <v>19</v>
       </c>
       <c r="D17" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E17" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G17" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H17">
         <v>100</v>
       </c>
       <c r="I17" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="J17" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -1406,25 +1409,25 @@
         <v>19</v>
       </c>
       <c r="D18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E18" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G18" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H18">
         <v>100</v>
       </c>
       <c r="I18" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="J18" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -1438,22 +1441,22 @@
         <v>19</v>
       </c>
       <c r="D19" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E19" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G19" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H19">
         <v>100</v>
       </c>
       <c r="I19" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -1467,25 +1470,25 @@
         <v>19</v>
       </c>
       <c r="D20" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E20" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F20" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G20" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H20">
         <v>100</v>
       </c>
       <c r="I20" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="K20" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -1499,28 +1502,25 @@
         <v>19</v>
       </c>
       <c r="D21" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E21" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F21" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G21" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H21">
         <v>30</v>
       </c>
       <c r="I21" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="J21" t="s">
-        <v>157</v>
-      </c>
-      <c r="K21" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -1534,22 +1534,22 @@
         <v>19</v>
       </c>
       <c r="D22" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E22" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G22" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H22">
         <v>100</v>
       </c>
       <c r="I22" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="23" spans="1:11">
@@ -1563,22 +1563,22 @@
         <v>20</v>
       </c>
       <c r="D23" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E23" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F23" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G23" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H23">
         <v>100</v>
       </c>
       <c r="I23" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -1592,25 +1592,25 @@
         <v>20</v>
       </c>
       <c r="D24" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E24" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F24" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G24" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H24">
         <v>35</v>
       </c>
       <c r="I24" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="J24" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -1624,16 +1624,16 @@
         <v>20</v>
       </c>
       <c r="D25" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E25" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F25" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G25" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H25">
         <v>100</v>
@@ -1653,25 +1653,25 @@
         <v>20</v>
       </c>
       <c r="D26" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E26" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F26" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G26" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H26">
         <v>50</v>
       </c>
       <c r="I26" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="J26" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="27" spans="1:11">
@@ -1685,16 +1685,16 @@
         <v>20</v>
       </c>
       <c r="D27" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E27" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F27" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G27" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H27">
         <v>100</v>
@@ -1714,22 +1714,22 @@
         <v>20</v>
       </c>
       <c r="D28" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E28" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F28" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G28" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H28">
         <v>50</v>
       </c>
       <c r="I28" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="29" spans="1:11">
@@ -1743,16 +1743,16 @@
         <v>21</v>
       </c>
       <c r="D29" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E29" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F29" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G29" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H29">
         <v>100</v>
@@ -1761,7 +1761,7 @@
         <v>21</v>
       </c>
       <c r="J29" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="30" spans="1:11">
@@ -1775,16 +1775,16 @@
         <v>21</v>
       </c>
       <c r="D30" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E30" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F30" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G30" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H30">
         <v>100</v>
@@ -1804,22 +1804,22 @@
         <v>21</v>
       </c>
       <c r="D31" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E31" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F31" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G31" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H31">
         <v>100</v>
       </c>
       <c r="I31" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -1833,22 +1833,22 @@
         <v>21</v>
       </c>
       <c r="D32" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E32" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F32" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G32" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H32">
         <v>100</v>
       </c>
       <c r="I32" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="33" spans="1:11">
@@ -1862,22 +1862,22 @@
         <v>21</v>
       </c>
       <c r="D33" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E33" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F33" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G33" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H33">
         <v>100</v>
       </c>
       <c r="I33" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="34" spans="1:11">
@@ -1891,25 +1891,25 @@
         <v>22</v>
       </c>
       <c r="D34" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E34" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F34" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G34" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H34">
         <v>100</v>
       </c>
       <c r="I34" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="J34" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="35" spans="1:11">
@@ -1923,25 +1923,25 @@
         <v>22</v>
       </c>
       <c r="D35" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E35" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F35" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G35" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H35">
         <v>50</v>
       </c>
       <c r="I35" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J35" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -1955,25 +1955,25 @@
         <v>23</v>
       </c>
       <c r="D36" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E36" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F36" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G36" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H36">
         <v>100</v>
       </c>
       <c r="I36" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="J36" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="37" spans="1:11">
@@ -1987,22 +1987,22 @@
         <v>23</v>
       </c>
       <c r="D37" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E37" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F37" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G37" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H37">
         <v>100</v>
       </c>
       <c r="I37" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="38" spans="1:11">
@@ -2016,25 +2016,25 @@
         <v>23</v>
       </c>
       <c r="D38" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E38" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F38" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G38" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H38">
         <v>50</v>
       </c>
       <c r="I38" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="J38" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="39" spans="1:11">
@@ -2048,25 +2048,25 @@
         <v>24</v>
       </c>
       <c r="D39" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E39" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F39" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G39" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H39">
         <v>100</v>
       </c>
       <c r="I39" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="J39" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="40" spans="1:11">
@@ -2080,22 +2080,22 @@
         <v>23</v>
       </c>
       <c r="D40" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E40" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F40" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G40" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H40">
         <v>100</v>
       </c>
       <c r="I40" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="41" spans="1:11">
@@ -2109,22 +2109,22 @@
         <v>23</v>
       </c>
       <c r="D41" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E41" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F41" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G41" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H41">
         <v>0</v>
       </c>
       <c r="I41" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="42" spans="1:11">
@@ -2138,28 +2138,28 @@
         <v>23</v>
       </c>
       <c r="D42" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E42" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F42" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G42" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H42">
         <v>100</v>
       </c>
       <c r="I42" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="J42" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="K42" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="43" spans="1:11">
@@ -2173,25 +2173,25 @@
         <v>23</v>
       </c>
       <c r="D43" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E43" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F43" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G43" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H43">
         <v>100</v>
       </c>
       <c r="I43" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="J43" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="44" spans="1:11">
@@ -2205,22 +2205,22 @@
         <v>23</v>
       </c>
       <c r="D44" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E44" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F44" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G44" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H44">
         <v>100</v>
       </c>
       <c r="I44" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="45" spans="1:11">
@@ -2234,25 +2234,25 @@
         <v>23</v>
       </c>
       <c r="D45" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E45" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F45" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G45" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H45">
         <v>0</v>
       </c>
       <c r="I45" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="J45" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="46" spans="1:11">
@@ -2266,25 +2266,25 @@
         <v>25</v>
       </c>
       <c r="D46" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E46" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F46" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G46" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H46">
         <v>100</v>
       </c>
       <c r="I46" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="J46" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="47" spans="1:11">
@@ -2298,22 +2298,22 @@
         <v>25</v>
       </c>
       <c r="D47" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E47" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F47" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G47" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H47">
         <v>100</v>
       </c>
       <c r="I47" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="48" spans="1:11">
@@ -2327,22 +2327,22 @@
         <v>25</v>
       </c>
       <c r="D48" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E48" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F48" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G48" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H48">
         <v>100</v>
       </c>
       <c r="I48" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="49" spans="1:10">
@@ -2356,22 +2356,22 @@
         <v>25</v>
       </c>
       <c r="D49" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E49" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F49" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G49" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H49">
         <v>100</v>
       </c>
       <c r="I49" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="50" spans="1:10">
@@ -2385,25 +2385,25 @@
         <v>25</v>
       </c>
       <c r="D50" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E50" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F50" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G50" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H50">
         <v>100</v>
       </c>
       <c r="I50" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="J50" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="51" spans="1:10">
@@ -2417,16 +2417,16 @@
         <v>25</v>
       </c>
       <c r="D51" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E51" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G51" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H51">
         <v>100</v>
@@ -2446,16 +2446,16 @@
         <v>26</v>
       </c>
       <c r="D52" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E52" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F52" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G52" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H52">
         <v>100</v>
@@ -2464,7 +2464,7 @@
         <v>26</v>
       </c>
       <c r="J52" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="53" spans="1:10">
@@ -2478,16 +2478,16 @@
         <v>27</v>
       </c>
       <c r="D53" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E53" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F53" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G53" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H53">
         <v>100</v>
@@ -2507,22 +2507,22 @@
         <v>27</v>
       </c>
       <c r="D54" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E54" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F54" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G54" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H54">
         <v>0</v>
       </c>
       <c r="I54" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="55" spans="1:10">
@@ -2536,22 +2536,22 @@
         <v>27</v>
       </c>
       <c r="D55" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E55" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F55" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G55" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H55">
         <v>100</v>
       </c>
       <c r="I55" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="56" spans="1:10">
@@ -2565,22 +2565,22 @@
         <v>27</v>
       </c>
       <c r="D56" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E56" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F56" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G56" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H56">
         <v>100</v>
       </c>
       <c r="I56" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="57" spans="1:10">
@@ -2594,22 +2594,22 @@
         <v>27</v>
       </c>
       <c r="D57" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E57" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F57" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G57" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H57">
         <v>100</v>
       </c>
       <c r="I57" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="58" spans="1:10">
@@ -2623,22 +2623,22 @@
         <v>27</v>
       </c>
       <c r="D58" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E58" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F58" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G58" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H58">
         <v>0</v>
       </c>
       <c r="I58" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="59" spans="1:10">
@@ -2652,22 +2652,22 @@
         <v>27</v>
       </c>
       <c r="D59" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E59" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F59" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G59" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H59">
         <v>50</v>
       </c>
       <c r="I59" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="60" spans="1:10">
@@ -2681,22 +2681,22 @@
         <v>27</v>
       </c>
       <c r="D60" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E60" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F60" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G60" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H60">
         <v>50</v>
       </c>
       <c r="I60" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="61" spans="1:10">
@@ -2710,16 +2710,16 @@
         <v>27</v>
       </c>
       <c r="D61" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E61" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F61" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G61" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H61">
         <v>100</v>
@@ -2728,7 +2728,7 @@
         <v>27</v>
       </c>
       <c r="J61" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="62" spans="1:10">
@@ -2742,22 +2742,22 @@
         <v>27</v>
       </c>
       <c r="D62" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E62" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F62" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G62" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H62">
         <v>100</v>
       </c>
       <c r="I62" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="63" spans="1:10">
@@ -2771,22 +2771,22 @@
         <v>27</v>
       </c>
       <c r="D63" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E63" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F63" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G63" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H63">
         <v>100</v>
       </c>
       <c r="I63" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="64" spans="1:10">
@@ -2800,22 +2800,22 @@
         <v>27</v>
       </c>
       <c r="D64" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E64" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F64" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G64" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H64">
         <v>0</v>
       </c>
       <c r="I64" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="65" spans="1:11">
@@ -2829,22 +2829,22 @@
         <v>27</v>
       </c>
       <c r="D65" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E65" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F65" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G65" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H65">
         <v>0</v>
       </c>
       <c r="I65" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="66" spans="1:11">
@@ -2858,22 +2858,22 @@
         <v>27</v>
       </c>
       <c r="D66" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E66" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F66" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G66" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H66">
         <v>0</v>
       </c>
       <c r="I66" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="67" spans="1:11">
@@ -2887,22 +2887,22 @@
         <v>27</v>
       </c>
       <c r="D67" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E67" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F67" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G67" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H67">
         <v>100</v>
       </c>
       <c r="I67" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="68" spans="1:11">
@@ -2916,22 +2916,22 @@
         <v>27</v>
       </c>
       <c r="D68" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E68" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F68" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G68" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H68">
         <v>50</v>
       </c>
       <c r="I68" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="69" spans="1:11">
@@ -2945,22 +2945,22 @@
         <v>27</v>
       </c>
       <c r="D69" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E69" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F69" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G69" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H69">
         <v>85</v>
       </c>
       <c r="I69" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="70" spans="1:11">
@@ -2974,16 +2974,16 @@
         <v>28</v>
       </c>
       <c r="D70" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E70" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F70" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G70" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H70">
         <v>100</v>
@@ -2992,7 +2992,7 @@
         <v>29</v>
       </c>
       <c r="K70" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="71" spans="1:11">
@@ -3006,16 +3006,16 @@
         <v>28</v>
       </c>
       <c r="D71" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E71" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F71" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G71" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H71">
         <v>100</v>
@@ -3035,22 +3035,22 @@
         <v>28</v>
       </c>
       <c r="D72" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E72" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F72" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G72" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H72">
         <v>100</v>
       </c>
       <c r="I72" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="73" spans="1:11">
@@ -3064,22 +3064,22 @@
         <v>28</v>
       </c>
       <c r="D73" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E73" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F73" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G73" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H73">
         <v>100</v>
       </c>
       <c r="I73" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="74" spans="1:11">
@@ -3093,22 +3093,22 @@
         <v>28</v>
       </c>
       <c r="D74" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E74" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F74" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G74" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H74">
         <v>100</v>
       </c>
       <c r="I74" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="75" spans="1:11">
@@ -3122,22 +3122,22 @@
         <v>29</v>
       </c>
       <c r="D75" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E75" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F75" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G75" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H75">
         <v>100</v>
       </c>
       <c r="I75" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="76" spans="1:11">
@@ -3151,22 +3151,22 @@
         <v>29</v>
       </c>
       <c r="D76" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E76" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F76" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G76" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H76">
         <v>100</v>
       </c>
       <c r="I76" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="77" spans="1:11">
@@ -3180,22 +3180,22 @@
         <v>29</v>
       </c>
       <c r="D77" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E77" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F77" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G77" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H77">
         <v>50</v>
       </c>
       <c r="I77" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="78" spans="1:11">
@@ -3209,22 +3209,22 @@
         <v>30</v>
       </c>
       <c r="D78" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E78" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F78" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G78" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H78">
         <v>100</v>
       </c>
       <c r="I78" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="79" spans="1:11">
@@ -3238,22 +3238,22 @@
         <v>31</v>
       </c>
       <c r="D79" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E79" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F79" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G79" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H79">
         <v>0</v>
       </c>
       <c r="I79" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="80" spans="1:11">
@@ -3267,22 +3267,51 @@
         <v>31</v>
       </c>
       <c r="D80" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E80" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F80" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G80" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H80">
         <v>0</v>
       </c>
       <c r="I80" t="s">
-        <v>150</v>
+        <v>152</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81" t="s">
+        <v>16</v>
+      </c>
+      <c r="C81" t="s">
+        <v>32</v>
+      </c>
+      <c r="D81" t="s">
+        <v>33</v>
+      </c>
+      <c r="E81" t="s">
+        <v>39</v>
+      </c>
+      <c r="F81" t="s">
+        <v>47</v>
+      </c>
+      <c r="G81" t="s">
+        <v>130</v>
+      </c>
+      <c r="H81">
+        <v>0</v>
+      </c>
+      <c r="I81" t="s">
+        <v>136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-06-23 00:42:08)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -4079,49 +4079,49 @@
       <c r="K78" s="1" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" t="n">
+      <c r="A79" s="3" t="n">
         <v>78</v>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="B79" s="3" t="inlineStr">
         <is>
           <t>Dirección</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
+      <c r="C79" s="3" t="inlineStr">
         <is>
           <t>16-Jun-26</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr">
+      <c r="F79" s="3" t="inlineStr">
         <is>
           <t>✂️ Corte</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr">
+      <c r="G79" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Definición de ACRONIMO y DISEÑO de orden de trabajo para Corte LASER. </t>
         </is>
       </c>
-      <c r="H79" t="n">
+      <c r="H79" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I79" t="inlineStr">
+      <c r="I79" s="3" t="inlineStr">
         <is>
           <t>23-Jun-26</t>
         </is>
       </c>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
+      <c r="J79" s="3" t="inlineStr"/>
+      <c r="K79" s="3" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="3" t="n">

</xml_diff>

<commit_message>
Sincronizacion MCE Planta (2026-06-24 19:28:58)
</commit_message>
<xml_diff>
--- a/base_matriz_mce.xlsx
+++ b/base_matriz_mce.xlsx
@@ -1628,53 +1628,53 @@
       <c r="K25" s="1" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" t="n">
+      <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>12-May-26</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>Jesús Morales</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>👑 Dirección</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>Autorización de Escritorios y Sillas</t>
         </is>
       </c>
-      <c r="H26" t="n">
+      <c r="H26" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>31-Jun-26</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
         <is>
           <t>28/May - Se a reenviado las Requisiciones al Ing. Alfredo para autorización 21348-21092</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -2045,53 +2045,53 @@
       <c r="K34" s="1" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="n">
+      <c r="A35" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>Auto Asignado</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>25-May-26</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>Jesús Morales</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>👑 Dirección</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>Solicitud de Computadora para Rodolfo Ingenieria</t>
         </is>
       </c>
-      <c r="H35" t="n">
+      <c r="H35" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="I35" s="2" t="inlineStr">
         <is>
           <t>5-Jun-2026</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="J35" s="2" t="inlineStr">
         <is>
           <t>28/May - Solicitud eviada al Ing. Alfredo de PC para Ing. Rodolfo.</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -2188,53 +2188,53 @@
       <c r="K37" s="1" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" t="n">
+      <c r="A38" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>Programa de Actividades</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F38" s="3" t="inlineStr">
         <is>
           <t>✂️ Corte</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="G38" s="3" t="inlineStr">
         <is>
           <t>Delimitar area de precausion de Maquina Lijadora (Negro-Amarillo)</t>
         </is>
       </c>
-      <c r="H38" t="n">
+      <c r="H38" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="I38" s="3" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="J38" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Quedamos a espera de la llegada de pintura color Negro/Amarillo </t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
+      <c r="K38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -2331,49 +2331,49 @@
       <c r="K40" s="1" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" t="n">
+      <c r="A41" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>Mejoras</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr">
         <is>
           <t>Bryan Flores</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" s="3" t="inlineStr">
         <is>
           <t>⚙️ Ingeniería</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>Capacitar en el uso de PRONEST</t>
         </is>
       </c>
-      <c r="H41" t="n">
+      <c r="H41" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="I41" s="3" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
+      <c r="J41" s="3" t="inlineStr"/>
+      <c r="K41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
@@ -4169,94 +4169,94 @@
       <c r="K80" s="3" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" t="n">
+      <c r="A81" s="1" t="n">
         <v>80</v>
       </c>
-      <c r="B81" t="inlineStr">
+      <c r="B81" s="1" t="inlineStr">
         <is>
           <t>Dirección</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="C81" s="1" t="inlineStr">
         <is>
           <t>22-Jun-26</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
+      <c r="D81" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E81" s="1" t="inlineStr">
         <is>
           <t>Jesús Morales</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr">
+      <c r="F81" s="1" t="inlineStr">
         <is>
           <t>👑 Dirección</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr">
+      <c r="G81" s="1" t="inlineStr">
         <is>
           <t>Actualización de APP, Mejoras con Imagen Corporativa.</t>
         </is>
       </c>
-      <c r="H81" t="n">
-        <v>0</v>
-      </c>
-      <c r="I81" t="inlineStr">
+      <c r="H81" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I81" s="1" t="inlineStr">
         <is>
           <t>27-Jun-26</t>
         </is>
       </c>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr"/>
+      <c r="J81" s="1" t="inlineStr"/>
+      <c r="K81" s="1" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" t="n">
+      <c r="A82" s="1" t="n">
         <v>81</v>
       </c>
-      <c r="B82" t="inlineStr">
+      <c r="B82" s="1" t="inlineStr">
         <is>
           <t>Dirección</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="C82" s="1" t="inlineStr">
         <is>
           <t>22-Jun-26</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
+      <c r="D82" s="1" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E82" s="1" t="inlineStr">
         <is>
           <t>Jesús Morales</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr">
+      <c r="F82" s="1" t="inlineStr">
         <is>
           <t>👥 Recursos Humanos</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr">
+      <c r="G82" s="1" t="inlineStr">
         <is>
           <t>Actualización de APP, Mejoras con Imagen Corporativa.</t>
         </is>
       </c>
-      <c r="H82" t="n">
-        <v>0</v>
-      </c>
-      <c r="I82" t="inlineStr">
+      <c r="H82" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I82" s="1" t="inlineStr">
         <is>
           <t>27-Jun-26</t>
         </is>
       </c>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr"/>
+      <c r="J82" s="1" t="inlineStr"/>
+      <c r="K82" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>